<commit_message>
chihan paati complete and kali mai mandir complete
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/नगर बजेट estimate/कालिकामाई मन्दिर पूर्वाधार विकास/कालिकामाई मन्दिर पूर्वाधार विकास.xlsx
+++ b/बजेट माग estimate/नगर बजेट estimate/कालिकामाई मन्दिर पूर्वाधार विकास/कालिकामाई मन्दिर पूर्वाधार विकास.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F66ACE7E-08EF-420B-9195-30C64B44A44D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24A0467-1D26-4224-9028-2F0F9B370EEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <definedName name="description_781">#REF!</definedName>
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="description_784">[3]Abstract!$B$300</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$55</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$88</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">estimate!$1:$8</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="69">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -204,6 +204,75 @@
   </si>
   <si>
     <t>rm</t>
+  </si>
+  <si>
+    <t>Earthwork Excavation in Cutting., Roadway Excavation in all types of Soil by Manual Means ., Roadway Excavation in all types of soil as per drawing and technical specification, including removal of stumps and other deleterious matter, with all lifts and lead as per Drawing and instruction of the Engineer.</t>
+  </si>
+  <si>
+    <t>-for levelling</t>
+  </si>
+  <si>
+    <t>-for steps</t>
+  </si>
+  <si>
+    <t>-Area for brick wall</t>
+  </si>
+  <si>
+    <t>-for flooring</t>
+  </si>
+  <si>
+    <t>sqm</t>
+  </si>
+  <si>
+    <t>dfn;fdfg pknAw u/L %) dL=dL= df]6f] x]eL 8o"6L OG6/nls+u s+lqm6Ans %) dL=dL=df]6fOsf] qm;/ 8:6 dfyL /fvL la5ofpg]] sfd k'/f .</t>
+  </si>
+  <si>
+    <t>-13% VAT for grey interlocking block</t>
+  </si>
+  <si>
+    <t>-13% VAT for stone dust (area*5cm)</t>
+  </si>
+  <si>
+    <t>-13% VAT for stone dust</t>
+  </si>
+  <si>
+    <t>e'O{+tNnfdf lrDgL e§fsf] O{+6fsf] uf/f] l;d]G6 d;nf -!M^_ df</t>
+  </si>
+  <si>
+    <t>-for brick wall</t>
+  </si>
+  <si>
+    <t>cum</t>
+  </si>
+  <si>
+    <t>-13% VAT for brick</t>
+  </si>
+  <si>
+    <t>sfnf] kmnfd] kfO{ksf] 6«; agfO{ h8fg ug]{ sfd</t>
+  </si>
+  <si>
+    <t>Length (m)</t>
+  </si>
+  <si>
+    <t>Unit Weight (kg/m)</t>
+  </si>
+  <si>
+    <t>Total Weight (Kg)</t>
+  </si>
+  <si>
+    <t>-Rectangular hollow section of size 80mm*40mm*1.6mm for diyo works around temple</t>
+  </si>
+  <si>
+    <t>- MS Square pipe of size 3"*3" with 1.6mm thickness for post</t>
+  </si>
+  <si>
+    <t>Kg</t>
+  </si>
+  <si>
+    <t>Provisional sum for unforseen works</t>
+  </si>
+  <si>
+    <t>PS</t>
   </si>
 </sst>
 </file>
@@ -279,6 +348,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -384,7 +454,7 @@
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -474,23 +544,8 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -511,10 +566,34 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1044,7 +1123,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:S55"/>
+  <dimension ref="A1:S88"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.7109375" style="19" customWidth="1"/>
@@ -1063,113 +1142,113 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
     </row>
     <row r="2" spans="1:16" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="40"/>
-      <c r="C2" s="40"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="I2" s="48"/>
+      <c r="J2" s="48"/>
+      <c r="K2" s="48"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49"/>
+      <c r="I3" s="49"/>
+      <c r="J3" s="49"/>
+      <c r="K3" s="49"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="41"/>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="41"/>
-      <c r="K4" s="41"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
+      <c r="G4" s="49"/>
+      <c r="H4" s="49"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="49"/>
+      <c r="K4" s="49"/>
     </row>
     <row r="5" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="42"/>
-      <c r="K5" s="42"/>
+      <c r="B5" s="50"/>
+      <c r="C5" s="50"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="50"/>
+      <c r="G5" s="50"/>
+      <c r="H5" s="50"/>
+      <c r="I5" s="50"/>
+      <c r="J5" s="50"/>
+      <c r="K5" s="50"/>
     </row>
     <row r="6" spans="1:16" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="37"/>
-      <c r="C6" s="37"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="37"/>
-      <c r="F6" s="37"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="38" t="s">
+      <c r="H6" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="38"/>
-      <c r="J6" s="38"/>
-      <c r="K6" s="38"/>
+      <c r="I6" s="46"/>
+      <c r="J6" s="46"/>
+      <c r="K6" s="46"/>
     </row>
     <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="45"/>
-      <c r="C7" s="45"/>
-      <c r="D7" s="45"/>
-      <c r="E7" s="45"/>
-      <c r="F7" s="45"/>
+      <c r="B7" s="40"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="46" t="s">
+      <c r="H7" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="I7" s="46"/>
-      <c r="J7" s="46"/>
-      <c r="K7" s="46"/>
+      <c r="I7" s="41"/>
+      <c r="J7" s="41"/>
+      <c r="K7" s="41"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
@@ -1206,12 +1285,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="150" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="180" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="16">
         <v>1</v>
       </c>
-      <c r="B9" s="50" t="s">
-        <v>42</v>
+      <c r="B9" s="35" t="s">
+        <v>46</v>
       </c>
       <c r="C9" s="17"/>
       <c r="D9" s="17"/>
@@ -1226,19 +1305,23 @@
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="32" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C10" s="17">
         <v>1</v>
       </c>
       <c r="D10" s="33">
-        <v>15</v>
-      </c>
-      <c r="E10" s="33"/>
-      <c r="F10" s="33"/>
+        <v>2</v>
+      </c>
+      <c r="E10" s="33">
+        <v>2.7</v>
+      </c>
+      <c r="F10" s="33">
+        <v>0.15</v>
+      </c>
       <c r="G10" s="33">
         <f>PRODUCT(C10:F10)</f>
-        <v>15</v>
+        <v>0.81</v>
       </c>
       <c r="H10" s="17"/>
       <c r="I10" s="17"/>
@@ -1258,216 +1341,254 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="34" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="6">
-        <f>SUM(G10:G10)</f>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" s="16"/>
+      <c r="B11" s="32"/>
+      <c r="C11" s="17">
+        <v>1</v>
+      </c>
+      <c r="D11" s="33">
+        <f>15</f>
         <v>15</v>
       </c>
-      <c r="H11" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="I11" s="6">
-        <v>4132.8</v>
-      </c>
-      <c r="J11" s="18">
-        <f>G11*I11</f>
-        <v>61992</v>
-      </c>
-      <c r="K11" s="5"/>
+      <c r="E11" s="33">
+        <v>3.4</v>
+      </c>
+      <c r="F11" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G11" s="33">
+        <f t="shared" ref="G11:G13" si="0">PRODUCT(C11:F11)</f>
+        <v>7.6499999999999995</v>
+      </c>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
+      <c r="M11" s="51"/>
+      <c r="N11" s="51"/>
+      <c r="O11" s="51"/>
+      <c r="P11" s="51"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
       <c r="B12" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
+        <v>48</v>
+      </c>
+      <c r="C12" s="17">
+        <v>1</v>
+      </c>
+      <c r="D12" s="33">
+        <f>1.5+D17</f>
+        <v>7.5957025297165499</v>
+      </c>
+      <c r="E12" s="33">
+        <v>1.2</v>
+      </c>
+      <c r="F12" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G12" s="33">
+        <f t="shared" si="0"/>
+        <v>1.3672264553489788</v>
+      </c>
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
-      <c r="J12" s="18">
-        <f>0.13*J11</f>
-        <v>8058.96</v>
-      </c>
+      <c r="J12" s="17"/>
       <c r="K12" s="17"/>
+      <c r="M12" s="36"/>
+      <c r="N12" s="36"/>
+      <c r="O12" s="36"/>
+      <c r="P12" s="36"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
+      <c r="B13" s="32" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="17">
+        <v>1</v>
+      </c>
+      <c r="D13" s="33">
+        <v>4</v>
+      </c>
+      <c r="E13" s="33">
+        <v>0.23</v>
+      </c>
+      <c r="F13" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G13" s="33">
+        <f t="shared" si="0"/>
+        <v>0.13800000000000001</v>
+      </c>
       <c r="H13" s="17"/>
       <c r="I13" s="17"/>
       <c r="J13" s="17"/>
       <c r="K13" s="17"/>
-    </row>
-    <row r="14" spans="1:16" ht="188.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="16">
-        <v>1</v>
-      </c>
-      <c r="B14" s="35" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
+      <c r="M13" s="36"/>
+      <c r="N13" s="36"/>
+      <c r="O13" s="36"/>
+      <c r="P13" s="36"/>
+    </row>
+    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+      <c r="B14" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="6">
+        <f>SUM(G10:G13)</f>
+        <v>9.9652264553489776</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I14" s="6">
+        <v>748.9</v>
+      </c>
+      <c r="J14" s="18">
+        <f>G14*I14</f>
+        <v>7462.9580924108486</v>
+      </c>
+      <c r="K14" s="5"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
-      <c r="B15" s="32" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="17">
-        <v>1</v>
-      </c>
-      <c r="D15" s="33">
-        <v>18.5</v>
-      </c>
-      <c r="E15" s="33">
-        <f>F15/2</f>
-        <v>1.5</v>
-      </c>
-      <c r="F15" s="33">
-        <v>3</v>
-      </c>
-      <c r="G15" s="33">
-        <f>PRODUCT(C15:F15)</f>
-        <v>83.25</v>
-      </c>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
       <c r="H15" s="17"/>
       <c r="I15" s="17"/>
       <c r="J15" s="17"/>
       <c r="K15" s="17"/>
-      <c r="M15" s="33">
-        <f>7</f>
-        <v>7</v>
-      </c>
-      <c r="N15" s="33">
-        <f>2</f>
+    </row>
+    <row r="16" spans="1:16" ht="188.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="16">
         <v>2</v>
       </c>
-      <c r="O15" s="33"/>
-      <c r="P15" s="33">
-        <f>PI()*M15*SQRT(M15^2+N15^2)</f>
-        <v>160.09797821843054</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A16" s="16"/>
-      <c r="B16" s="32"/>
+      <c r="B16" s="35" t="s">
+        <v>39</v>
+      </c>
       <c r="C16" s="17"/>
-      <c r="D16" s="33"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="33"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
       <c r="J16" s="17"/>
       <c r="K16" s="17"/>
-      <c r="M16" s="51"/>
-      <c r="N16" s="51"/>
-      <c r="O16" s="51"/>
-      <c r="P16" s="51"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="16"/>
-      <c r="B17" s="32"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
+      <c r="B17" s="32" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="17">
+        <v>1</v>
+      </c>
+      <c r="D17" s="33">
+        <f>D22</f>
+        <v>6.0957025297165499</v>
+      </c>
+      <c r="E17" s="33">
+        <f>E22</f>
+        <v>1.925</v>
+      </c>
+      <c r="F17" s="33">
+        <v>0.75</v>
+      </c>
+      <c r="G17" s="33">
+        <f>PRODUCT(C17:F17)</f>
+        <v>8.8006705272782693</v>
+      </c>
       <c r="H17" s="17"/>
       <c r="I17" s="17"/>
       <c r="J17" s="17"/>
       <c r="K17" s="17"/>
-      <c r="M17" s="51"/>
-      <c r="N17" s="51"/>
-      <c r="O17" s="51"/>
-      <c r="P17" s="51"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="16"/>
-      <c r="B18" s="32"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="33"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="33"/>
-      <c r="G18" s="33"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="M18" s="51"/>
-      <c r="N18" s="51"/>
-      <c r="O18" s="51"/>
-      <c r="P18" s="51"/>
+      <c r="M17" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N17" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O17" s="33"/>
+      <c r="P17" s="33">
+        <f>PI()*M17*SQRT(M17^2+N17^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+      <c r="B18" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" s="3"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="6">
+        <f>SUM(G17:G17)</f>
+        <v>8.8006705272782693</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I18" s="6">
+        <v>62.95</v>
+      </c>
+      <c r="J18" s="18">
+        <f>G18*I18</f>
+        <v>554.00220969216707</v>
+      </c>
+      <c r="K18" s="5"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="16"/>
-      <c r="B19" s="32"/>
+      <c r="B19" s="32" t="s">
+        <v>24</v>
+      </c>
       <c r="C19" s="17"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="33"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
       <c r="H19" s="17"/>
       <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
+      <c r="J19" s="18">
+        <f>0.13*G18*(18612)/360</f>
+        <v>59.149306613837254</v>
+      </c>
       <c r="K19" s="17"/>
-      <c r="M19" s="51"/>
-      <c r="N19" s="51"/>
-      <c r="O19" s="51"/>
-      <c r="P19" s="51"/>
-    </row>
-    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="34" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20" s="3"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="6">
-        <f>SUM(G15:G15)</f>
-        <v>83.25</v>
-      </c>
-      <c r="H20" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I20" s="6">
-        <v>62.95</v>
-      </c>
-      <c r="J20" s="18">
-        <f>G20*I20</f>
-        <v>5240.5875000000005</v>
-      </c>
-      <c r="K20" s="5"/>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A21" s="16"/>
-      <c r="B21" s="32" t="s">
-        <v>24</v>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A20" s="16"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
+    </row>
+    <row r="21" spans="1:16" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="16">
+        <v>3</v>
+      </c>
+      <c r="B21" s="35" t="s">
+        <v>31</v>
       </c>
       <c r="C21" s="17"/>
       <c r="D21" s="17"/>
@@ -1476,130 +1597,180 @@
       <c r="G21" s="17"/>
       <c r="H21" s="17"/>
       <c r="I21" s="17"/>
-      <c r="J21" s="18">
-        <f>0.13*G20*(18612)/360</f>
-        <v>559.52324999999996</v>
-      </c>
+      <c r="J21" s="17"/>
       <c r="K21" s="17"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="16"/>
-      <c r="B22" s="17"/>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
+      <c r="B22" s="32" t="str">
+        <f>B17</f>
+        <v>-for masonary wall</v>
+      </c>
+      <c r="C22" s="17">
+        <v>1</v>
+      </c>
+      <c r="D22" s="33">
+        <f>D30</f>
+        <v>6.0957025297165499</v>
+      </c>
+      <c r="E22" s="33">
+        <f>E30</f>
+        <v>1.925</v>
+      </c>
+      <c r="F22" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G22" s="33">
+        <f>PRODUCT(C22:F22)</f>
+        <v>1.7601341054556536</v>
+      </c>
       <c r="H22" s="17"/>
       <c r="I22" s="17"/>
       <c r="J22" s="17"/>
       <c r="K22" s="17"/>
-    </row>
-    <row r="23" spans="1:16" ht="94.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="16">
+      <c r="M22" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N22" s="33">
+        <f>2</f>
         <v>2</v>
       </c>
-      <c r="B23" s="35" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
+      <c r="O22" s="33"/>
+      <c r="P22" s="33">
+        <f>PI()*M22*SQRT(M22^2+N22^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" s="16"/>
+      <c r="B23" s="32" t="str">
+        <f>B10</f>
+        <v>-for levelling</v>
+      </c>
+      <c r="C23" s="17">
+        <f>C10</f>
+        <v>1</v>
+      </c>
+      <c r="D23" s="33">
+        <f>D10</f>
+        <v>2</v>
+      </c>
+      <c r="E23" s="33">
+        <f>E10</f>
+        <v>2.7</v>
+      </c>
+      <c r="F23" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G23" s="33">
+        <f t="shared" ref="G23:G25" si="1">PRODUCT(C23:F23)</f>
+        <v>0.81</v>
+      </c>
       <c r="H23" s="17"/>
       <c r="I23" s="17"/>
       <c r="J23" s="17"/>
       <c r="K23" s="17"/>
+      <c r="M23" s="51"/>
+      <c r="N23" s="51"/>
+      <c r="O23" s="51"/>
+      <c r="P23" s="51"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="16"/>
-      <c r="B24" s="32" t="str">
-        <f>B10</f>
-        <v>-for railing</v>
-      </c>
+      <c r="B24" s="32"/>
       <c r="C24" s="17">
+        <f>C11</f>
         <v>1</v>
       </c>
       <c r="D24" s="33">
-        <f>D10</f>
+        <f t="shared" ref="D24:E25" si="2">D11</f>
         <v>15</v>
       </c>
       <c r="E24" s="33">
-        <f>E10</f>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>3.4</v>
       </c>
       <c r="F24" s="33">
         <v>0.15</v>
       </c>
       <c r="G24" s="33">
-        <f>PRODUCT(C24:F24)</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>7.6499999999999995</v>
       </c>
       <c r="H24" s="17"/>
       <c r="I24" s="17"/>
       <c r="J24" s="17"/>
       <c r="K24" s="17"/>
-      <c r="M24" s="33">
-        <f>7</f>
-        <v>7</v>
-      </c>
-      <c r="N24" s="33">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="O24" s="33"/>
-      <c r="P24" s="33">
-        <f>PI()*M24*SQRT(M24^2+N24^2)</f>
-        <v>160.09797821843054</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="2"/>
-      <c r="B25" s="34" t="s">
+      <c r="M24" s="51"/>
+      <c r="N24" s="51"/>
+      <c r="O24" s="51"/>
+      <c r="P24" s="51"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="16"/>
+      <c r="B25" s="32" t="str">
+        <f t="shared" ref="B25" si="3">B12</f>
+        <v>-for steps</v>
+      </c>
+      <c r="C25" s="17">
+        <f>C12</f>
+        <v>1</v>
+      </c>
+      <c r="D25" s="33">
+        <f t="shared" si="2"/>
+        <v>7.5957025297165499</v>
+      </c>
+      <c r="E25" s="33">
+        <f t="shared" si="2"/>
+        <v>1.2</v>
+      </c>
+      <c r="F25" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G25" s="33">
+        <f t="shared" si="1"/>
+        <v>1.3672264553489788</v>
+      </c>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+      <c r="M25" s="51"/>
+      <c r="N25" s="51"/>
+      <c r="O25" s="51"/>
+      <c r="P25" s="51"/>
+    </row>
+    <row r="26" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2"/>
+      <c r="B26" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="C25" s="3"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="6">
-        <f>SUM(G24:G24)</f>
-        <v>0</v>
-      </c>
-      <c r="H25" s="7" t="s">
+      <c r="C26" s="3"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="6">
+        <f>SUM(G22:G25)</f>
+        <v>11.587360560804632</v>
+      </c>
+      <c r="H26" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="I25" s="6">
+      <c r="I26" s="6">
         <v>4458.5200000000004</v>
       </c>
-      <c r="J25" s="18">
-        <f>G25*I25</f>
-        <v>0</v>
-      </c>
-      <c r="K25" s="5"/>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="16"/>
-      <c r="B26" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
       <c r="J26" s="18">
-        <f>0.13*G25*(14817.6)/5</f>
-        <v>0</v>
-      </c>
-      <c r="K26" s="17"/>
+        <f>G26*I26</f>
+        <v>51662.478807558669</v>
+      </c>
+      <c r="K26" s="5"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="16"/>
-      <c r="B27" s="17"/>
+      <c r="B27" s="32" t="s">
+        <v>24</v>
+      </c>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
       <c r="E27" s="17"/>
@@ -1607,16 +1778,15 @@
       <c r="G27" s="17"/>
       <c r="H27" s="17"/>
       <c r="I27" s="17"/>
-      <c r="J27" s="17"/>
+      <c r="J27" s="18">
+        <f>0.13*G26*(14817.6)/5</f>
+        <v>4464.118719990247</v>
+      </c>
       <c r="K27" s="17"/>
     </row>
-    <row r="28" spans="1:16" ht="78.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="16">
-        <v>3</v>
-      </c>
-      <c r="B28" s="35" t="s">
-        <v>32</v>
-      </c>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="16"/>
+      <c r="B28" s="17"/>
       <c r="C28" s="17"/>
       <c r="D28" s="17"/>
       <c r="E28" s="17"/>
@@ -1627,195 +1797,256 @@
       <c r="J28" s="17"/>
       <c r="K28" s="17"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A29" s="16"/>
-      <c r="B29" s="32" t="str">
-        <f>B24</f>
-        <v>-for railing</v>
-      </c>
-      <c r="C29" s="17">
-        <v>1</v>
-      </c>
-      <c r="D29" s="33">
-        <f>D24</f>
-        <v>15</v>
-      </c>
-      <c r="E29" s="33">
-        <f>E24</f>
-        <v>0</v>
-      </c>
-      <c r="F29" s="33">
-        <v>0.05</v>
-      </c>
-      <c r="G29" s="33">
-        <f>PRODUCT(C29:F29)</f>
-        <v>0</v>
-      </c>
+    <row r="29" spans="1:16" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="16">
+        <v>4</v>
+      </c>
+      <c r="B29" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
       <c r="H29" s="17"/>
       <c r="I29" s="17"/>
       <c r="J29" s="17"/>
       <c r="K29" s="17"/>
-      <c r="M29" s="33">
-        <f>7</f>
-        <v>7</v>
-      </c>
-      <c r="N29" s="33">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="O29" s="33"/>
-      <c r="P29" s="33">
-        <f>PI()*M29*SQRT(M29^2+N29^2)</f>
-        <v>160.09797821843054</v>
-      </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
-      <c r="B30" s="32"/>
+      <c r="B30" s="32" t="str">
+        <f>B22</f>
+        <v>-for masonary wall</v>
+      </c>
       <c r="C30" s="17">
         <v>1</v>
       </c>
       <c r="D30" s="33">
-        <f>D29</f>
-        <v>15</v>
+        <f>D44</f>
+        <v>6.0957025297165499</v>
       </c>
       <c r="E30" s="33">
-        <v>0.45</v>
+        <f>F44/2</f>
+        <v>1.925</v>
       </c>
       <c r="F30" s="33">
         <v>0.05</v>
       </c>
       <c r="G30" s="33">
         <f>PRODUCT(C30:F30)</f>
-        <v>0.33750000000000002</v>
+        <v>0.58671136848521799</v>
       </c>
       <c r="H30" s="17"/>
       <c r="I30" s="17"/>
       <c r="J30" s="17"/>
       <c r="K30" s="17"/>
-      <c r="M30" s="36"/>
-      <c r="N30" s="36"/>
-      <c r="O30" s="36"/>
-      <c r="P30" s="36"/>
-    </row>
-    <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="2"/>
-      <c r="B31" s="34" t="s">
-        <v>17</v>
-      </c>
-      <c r="C31" s="3"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="6">
-        <f>SUM(G29:G30)</f>
-        <v>0.33750000000000002</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I31" s="6">
-        <v>10964.46</v>
-      </c>
-      <c r="J31" s="18">
-        <f>G31*I31</f>
-        <v>3700.5052500000002</v>
-      </c>
-      <c r="K31" s="5"/>
+      <c r="M30" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N30" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O30" s="33"/>
+      <c r="P30" s="33">
+        <f>PI()*M30*SQRT(M30^2+N30^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" s="16"/>
+      <c r="B31" s="32"/>
+      <c r="C31" s="17">
+        <v>1</v>
+      </c>
+      <c r="D31" s="33">
+        <f>D30</f>
+        <v>6.0957025297165499</v>
+      </c>
+      <c r="E31" s="33">
+        <v>0.45</v>
+      </c>
+      <c r="F31" s="33">
+        <v>0.05</v>
+      </c>
+      <c r="G31" s="33">
+        <f>PRODUCT(C31:F31)</f>
+        <v>0.13715330691862238</v>
+      </c>
+      <c r="H31" s="17"/>
+      <c r="I31" s="17"/>
+      <c r="J31" s="17"/>
+      <c r="K31" s="17"/>
+      <c r="M31" s="36"/>
+      <c r="N31" s="36"/>
+      <c r="O31" s="36"/>
+      <c r="P31" s="36"/>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="16"/>
-      <c r="B32" s="32" t="s">
-        <v>33</v>
-      </c>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
-      <c r="G32" s="17"/>
+      <c r="B32" s="32" t="str">
+        <f>B23</f>
+        <v>-for levelling</v>
+      </c>
+      <c r="C32" s="17">
+        <f>C23</f>
+        <v>1</v>
+      </c>
+      <c r="D32" s="33">
+        <f>D23</f>
+        <v>2</v>
+      </c>
+      <c r="E32" s="33">
+        <f>E23</f>
+        <v>2.7</v>
+      </c>
+      <c r="F32" s="33">
+        <v>0.05</v>
+      </c>
+      <c r="G32" s="33">
+        <f t="shared" ref="G32:G35" si="4">PRODUCT(C32:F32)</f>
+        <v>0.27</v>
+      </c>
       <c r="H32" s="17"/>
       <c r="I32" s="17"/>
-      <c r="J32" s="18">
-        <f>0.13*G31*(53818.03)/15</f>
-        <v>157.41773775000001</v>
-      </c>
+      <c r="J32" s="17"/>
       <c r="K32" s="17"/>
+      <c r="M32" s="36"/>
+      <c r="N32" s="36"/>
+      <c r="O32" s="36"/>
+      <c r="P32" s="36"/>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="16"/>
-      <c r="B33" s="32" t="s">
-        <v>34</v>
-      </c>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
+      <c r="B33" s="32"/>
+      <c r="C33" s="17">
+        <f t="shared" ref="C33:E33" si="5">C24</f>
+        <v>1</v>
+      </c>
+      <c r="D33" s="33">
+        <f t="shared" si="5"/>
+        <v>15</v>
+      </c>
+      <c r="E33" s="33">
+        <f t="shared" si="5"/>
+        <v>3.4</v>
+      </c>
+      <c r="F33" s="33">
+        <v>0.05</v>
+      </c>
+      <c r="G33" s="33">
+        <f t="shared" si="4"/>
+        <v>2.5500000000000003</v>
+      </c>
       <c r="H33" s="17"/>
       <c r="I33" s="17"/>
-      <c r="J33" s="18">
-        <f>0.13*G31*(21432.6)/15</f>
-        <v>62.690354999999997</v>
-      </c>
+      <c r="J33" s="17"/>
       <c r="K33" s="17"/>
+      <c r="M33" s="36"/>
+      <c r="N33" s="36"/>
+      <c r="O33" s="36"/>
+      <c r="P33" s="36"/>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="16"/>
-      <c r="B34" s="32" t="s">
-        <v>35</v>
-      </c>
-      <c r="C34" s="17"/>
-      <c r="D34" s="17"/>
-      <c r="E34" s="17"/>
-      <c r="F34" s="17"/>
-      <c r="G34" s="17"/>
+      <c r="B34" s="32" t="str">
+        <f>B25</f>
+        <v>-for steps</v>
+      </c>
+      <c r="C34" s="17">
+        <f t="shared" ref="C34:E34" si="6">C25</f>
+        <v>1</v>
+      </c>
+      <c r="D34" s="33">
+        <f t="shared" si="6"/>
+        <v>7.5957025297165499</v>
+      </c>
+      <c r="E34" s="33">
+        <f t="shared" si="6"/>
+        <v>1.2</v>
+      </c>
+      <c r="F34" s="33">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G34" s="33">
+        <f t="shared" si="4"/>
+        <v>0.6836132276744894</v>
+      </c>
       <c r="H34" s="17"/>
       <c r="I34" s="17"/>
-      <c r="J34" s="18">
-        <f>0.13*G31*(25719.12+13573.98+4286.52)/15</f>
-        <v>127.4703885</v>
-      </c>
+      <c r="J34" s="17"/>
       <c r="K34" s="17"/>
+      <c r="M34" s="36"/>
+      <c r="N34" s="36"/>
+      <c r="O34" s="36"/>
+      <c r="P34" s="36"/>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="16"/>
-      <c r="B35" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="17"/>
-      <c r="G35" s="17"/>
+      <c r="B35" s="32" t="str">
+        <f>B13</f>
+        <v>-Area for brick wall</v>
+      </c>
+      <c r="C35" s="17">
+        <f>C13</f>
+        <v>1</v>
+      </c>
+      <c r="D35" s="33">
+        <f>D13</f>
+        <v>4</v>
+      </c>
+      <c r="E35" s="33">
+        <v>0.23</v>
+      </c>
+      <c r="F35" s="33">
+        <v>0.05</v>
+      </c>
+      <c r="G35" s="33">
+        <f t="shared" si="4"/>
+        <v>4.6000000000000006E-2</v>
+      </c>
       <c r="H35" s="17"/>
       <c r="I35" s="17"/>
-      <c r="J35" s="18">
-        <f>0.13*G31*(6325.7)/15</f>
-        <v>18.502672500000003</v>
-      </c>
+      <c r="J35" s="17"/>
       <c r="K35" s="17"/>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A36" s="16"/>
-      <c r="B36" s="32" t="s">
-        <v>40</v>
-      </c>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="17"/>
-      <c r="F36" s="17"/>
-      <c r="G36" s="17"/>
-      <c r="H36" s="17"/>
-      <c r="I36" s="17"/>
+      <c r="M35" s="36"/>
+      <c r="N35" s="36"/>
+      <c r="O35" s="36"/>
+      <c r="P35" s="36"/>
+    </row>
+    <row r="36" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2"/>
+      <c r="B36" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C36" s="3"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="6">
+        <f>SUM(G30:G35)</f>
+        <v>4.2734779030783301</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I36" s="6">
+        <v>10964.46</v>
+      </c>
       <c r="J36" s="18">
-        <f>0.13*G31*(310)/5</f>
-        <v>2.7202500000000005</v>
-      </c>
-      <c r="K36" s="17"/>
+        <f>G36*I36</f>
+        <v>46856.377529186226</v>
+      </c>
+      <c r="K36" s="5"/>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="16"/>
-      <c r="B37" s="17"/>
+      <c r="B37" s="32" t="s">
+        <v>33</v>
+      </c>
       <c r="C37" s="17"/>
       <c r="D37" s="17"/>
       <c r="E37" s="17"/>
@@ -1823,15 +2054,16 @@
       <c r="G37" s="17"/>
       <c r="H37" s="17"/>
       <c r="I37" s="17"/>
-      <c r="J37" s="17"/>
+      <c r="J37" s="18">
+        <f>0.13*G36*(53818.03)/15</f>
+        <v>1993.2480705991243</v>
+      </c>
       <c r="K37" s="17"/>
     </row>
-    <row r="38" spans="1:16" ht="110.25" x14ac:dyDescent="0.25">
-      <c r="A38" s="16">
-        <v>4</v>
-      </c>
-      <c r="B38" s="35" t="s">
-        <v>37</v>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A38" s="16"/>
+      <c r="B38" s="32" t="s">
+        <v>34</v>
       </c>
       <c r="C38" s="17"/>
       <c r="D38" s="17"/>
@@ -1840,80 +2072,52 @@
       <c r="G38" s="17"/>
       <c r="H38" s="17"/>
       <c r="I38" s="17"/>
-      <c r="J38" s="17"/>
+      <c r="J38" s="18">
+        <f>0.13*G36*(21432.6)/15</f>
+        <v>793.79510171447725</v>
+      </c>
       <c r="K38" s="17"/>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="16"/>
-      <c r="B39" s="32" t="str">
-        <f>B29</f>
-        <v>-for railing</v>
-      </c>
-      <c r="C39" s="17">
-        <v>1</v>
-      </c>
-      <c r="D39" s="33">
-        <f>D10</f>
-        <v>15</v>
-      </c>
-      <c r="E39" s="33">
-        <f>((F39/2)+0.45)/2</f>
-        <v>0.97499999999999998</v>
-      </c>
-      <c r="F39" s="33">
-        <v>3</v>
-      </c>
-      <c r="G39" s="33">
-        <f>PRODUCT(C39:F39)</f>
-        <v>43.875</v>
-      </c>
+      <c r="B39" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="17"/>
+      <c r="G39" s="17"/>
       <c r="H39" s="17"/>
       <c r="I39" s="17"/>
-      <c r="J39" s="17"/>
+      <c r="J39" s="18">
+        <f>0.13*G36*(25719.12+13573.98+4286.52)/15</f>
+        <v>1614.0500401527704</v>
+      </c>
       <c r="K39" s="17"/>
-      <c r="M39" s="33">
-        <f>7</f>
-        <v>7</v>
-      </c>
-      <c r="N39" s="33">
-        <f>2</f>
-        <v>2</v>
-      </c>
-      <c r="O39" s="33"/>
-      <c r="P39" s="33">
-        <f>PI()*M39*SQRT(M39^2+N39^2)</f>
-        <v>160.09797821843054</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="2"/>
-      <c r="B40" s="34" t="s">
-        <v>17</v>
-      </c>
-      <c r="C40" s="3"/>
-      <c r="D40" s="4"/>
-      <c r="E40" s="5"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="6">
-        <f>SUM(G39:G39)</f>
-        <v>43.875</v>
-      </c>
-      <c r="H40" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="I40" s="6">
-        <v>8987.83</v>
-      </c>
+    </row>
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A40" s="16"/>
+      <c r="B40" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="C40" s="17"/>
+      <c r="D40" s="17"/>
+      <c r="E40" s="17"/>
+      <c r="F40" s="17"/>
+      <c r="G40" s="17"/>
+      <c r="H40" s="17"/>
+      <c r="I40" s="17"/>
       <c r="J40" s="18">
-        <f>G40*I40</f>
-        <v>394341.04125000001</v>
-      </c>
-      <c r="K40" s="5"/>
+        <f>0.13*G36*(6325.7)/15</f>
+        <v>234.28373948635578</v>
+      </c>
+      <c r="K40" s="17"/>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="16"/>
       <c r="B41" s="32" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C41" s="17"/>
       <c r="D41" s="17"/>
@@ -1923,16 +2127,14 @@
       <c r="H41" s="17"/>
       <c r="I41" s="17"/>
       <c r="J41" s="18">
-        <f>0.13*G40*(5863.95)/5</f>
-        <v>6689.3009625000004</v>
+        <f>0.13*G36*(310)/5</f>
+        <v>34.444231898811339</v>
       </c>
       <c r="K41" s="17"/>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="16"/>
-      <c r="B42" s="32" t="s">
-        <v>34</v>
-      </c>
+      <c r="B42" s="17"/>
       <c r="C42" s="17"/>
       <c r="D42" s="17"/>
       <c r="E42" s="17"/>
@@ -1940,16 +2142,15 @@
       <c r="G42" s="17"/>
       <c r="H42" s="17"/>
       <c r="I42" s="17"/>
-      <c r="J42" s="18">
-        <f>0.13*G40*(6604.416)/5</f>
-        <v>7533.9875520000005</v>
-      </c>
+      <c r="J42" s="17"/>
       <c r="K42" s="17"/>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A43" s="16"/>
-      <c r="B43" s="32" t="s">
-        <v>38</v>
+    <row r="43" spans="1:16" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="A43" s="16">
+        <v>5</v>
+      </c>
+      <c r="B43" s="35" t="s">
+        <v>37</v>
       </c>
       <c r="C43" s="17"/>
       <c r="D43" s="17"/>
@@ -1958,213 +2159,942 @@
       <c r="G43" s="17"/>
       <c r="H43" s="17"/>
       <c r="I43" s="17"/>
-      <c r="J43" s="18">
-        <f>0.13*G40*(14808.78)/5</f>
-        <v>16893.115785000002</v>
-      </c>
+      <c r="J43" s="17"/>
       <c r="K43" s="17"/>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" s="16"/>
-      <c r="B44" s="32" t="s">
-        <v>40</v>
-      </c>
-      <c r="C44" s="17"/>
-      <c r="D44" s="17"/>
-      <c r="E44" s="17"/>
-      <c r="F44" s="17"/>
-      <c r="G44" s="17"/>
+      <c r="B44" s="32" t="str">
+        <f>B30</f>
+        <v>-for masonary wall</v>
+      </c>
+      <c r="C44" s="17">
+        <v>1</v>
+      </c>
+      <c r="D44" s="33">
+        <f>20/3.281</f>
+        <v>6.0957025297165499</v>
+      </c>
+      <c r="E44" s="33">
+        <f>((F44/2)+0.45)/2</f>
+        <v>1.1875</v>
+      </c>
+      <c r="F44" s="33">
+        <v>3.85</v>
+      </c>
+      <c r="G44" s="33">
+        <f>PRODUCT(C44:F44)</f>
+        <v>27.868790003047852</v>
+      </c>
       <c r="H44" s="17"/>
       <c r="I44" s="17"/>
-      <c r="J44" s="18">
-        <f>0.13*G40*(310)/5</f>
-        <v>353.63250000000005</v>
-      </c>
+      <c r="J44" s="17"/>
       <c r="K44" s="17"/>
-    </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A45" s="16"/>
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="17"/>
-      <c r="K45" s="17"/>
-    </row>
-    <row r="46" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="2">
-        <v>5</v>
-      </c>
-      <c r="B46" s="1" t="s">
+      <c r="M44" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N44" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O44" s="33"/>
+      <c r="P44" s="33">
+        <f>PI()*M44*SQRT(M44^2+N44^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2"/>
+      <c r="B45" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C45" s="3"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+      <c r="G45" s="6">
+        <f>SUM(G44:G44)</f>
+        <v>27.868790003047852</v>
+      </c>
+      <c r="H45" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I45" s="6">
+        <v>8987.83</v>
+      </c>
+      <c r="J45" s="18">
+        <f>G45*I45</f>
+        <v>250479.94685309357</v>
+      </c>
+      <c r="K45" s="5"/>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A46" s="16"/>
+      <c r="B46" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="C46" s="17"/>
+      <c r="D46" s="17"/>
+      <c r="E46" s="17"/>
+      <c r="F46" s="17"/>
+      <c r="G46" s="17"/>
+      <c r="H46" s="17"/>
+      <c r="I46" s="17"/>
+      <c r="J46" s="18">
+        <f>0.13*G45*(5863.95)/5</f>
+        <v>4248.950969597684</v>
+      </c>
+      <c r="K46" s="17"/>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A47" s="16"/>
+      <c r="B47" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="C47" s="17"/>
+      <c r="D47" s="17"/>
+      <c r="E47" s="17"/>
+      <c r="F47" s="17"/>
+      <c r="G47" s="17"/>
+      <c r="H47" s="17"/>
+      <c r="I47" s="17"/>
+      <c r="J47" s="18">
+        <f>0.13*G45*(6604.416)/5</f>
+        <v>4785.4841475160019</v>
+      </c>
+      <c r="K47" s="17"/>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A48" s="16"/>
+      <c r="B48" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="C48" s="17"/>
+      <c r="D48" s="17"/>
+      <c r="E48" s="17"/>
+      <c r="F48" s="17"/>
+      <c r="G48" s="17"/>
+      <c r="H48" s="17"/>
+      <c r="I48" s="17"/>
+      <c r="J48" s="18">
+        <f>0.13*G45*(14808.78)/5</f>
+        <v>10730.272280554711</v>
+      </c>
+      <c r="K48" s="17"/>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A49" s="16"/>
+      <c r="B49" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="C49" s="17"/>
+      <c r="D49" s="17"/>
+      <c r="E49" s="17"/>
+      <c r="F49" s="17"/>
+      <c r="G49" s="17"/>
+      <c r="H49" s="17"/>
+      <c r="I49" s="17"/>
+      <c r="J49" s="18">
+        <f>0.13*G45*(310)/5</f>
+        <v>224.62244742456568</v>
+      </c>
+      <c r="K49" s="17"/>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A50" s="16"/>
+      <c r="B50" s="17"/>
+      <c r="C50" s="17"/>
+      <c r="D50" s="17"/>
+      <c r="E50" s="17"/>
+      <c r="F50" s="17"/>
+      <c r="G50" s="17"/>
+      <c r="H50" s="17"/>
+      <c r="I50" s="17"/>
+      <c r="J50" s="17"/>
+      <c r="K50" s="17"/>
+    </row>
+    <row r="51" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+      <c r="A51" s="16">
+        <v>6</v>
+      </c>
+      <c r="B51" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="C51" s="17"/>
+      <c r="D51" s="17"/>
+      <c r="E51" s="17"/>
+      <c r="F51" s="17"/>
+      <c r="G51" s="17"/>
+      <c r="H51" s="17"/>
+      <c r="I51" s="17"/>
+      <c r="J51" s="17"/>
+      <c r="K51" s="17"/>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A52" s="16"/>
+      <c r="B52" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="C52" s="17">
+        <v>1</v>
+      </c>
+      <c r="D52" s="33">
+        <f>D11</f>
+        <v>15</v>
+      </c>
+      <c r="E52" s="33">
+        <f>E11</f>
+        <v>3.4</v>
+      </c>
+      <c r="F52" s="33"/>
+      <c r="G52" s="33">
+        <f>PRODUCT(C52:F52)</f>
+        <v>51</v>
+      </c>
+      <c r="H52" s="17"/>
+      <c r="I52" s="17"/>
+      <c r="J52" s="17"/>
+      <c r="K52" s="17"/>
+      <c r="M52" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N52" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O52" s="33"/>
+      <c r="P52" s="33">
+        <f>PI()*M52*SQRT(M52^2+N52^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="2"/>
+      <c r="B53" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C53" s="3"/>
+      <c r="D53" s="4"/>
+      <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
+      <c r="G53" s="6">
+        <f>SUM(G52:G52)</f>
+        <v>51</v>
+      </c>
+      <c r="H53" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="I53" s="6">
+        <v>1754.28</v>
+      </c>
+      <c r="J53" s="18">
+        <f>G53*I53</f>
+        <v>89468.28</v>
+      </c>
+      <c r="K53" s="5"/>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A54" s="16"/>
+      <c r="B54" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="C54" s="17"/>
+      <c r="D54" s="17"/>
+      <c r="E54" s="17"/>
+      <c r="F54" s="17"/>
+      <c r="G54" s="17"/>
+      <c r="H54" s="17"/>
+      <c r="I54" s="17"/>
+      <c r="J54" s="18">
+        <f>0.13*G53*(6036.36/10)</f>
+        <v>4002.1066799999999</v>
+      </c>
+      <c r="K54" s="17"/>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A55" s="16"/>
+      <c r="B55" s="32" t="s">
+        <v>54</v>
+      </c>
+      <c r="C55" s="17"/>
+      <c r="D55" s="17"/>
+      <c r="E55" s="17"/>
+      <c r="F55" s="17"/>
+      <c r="G55" s="17"/>
+      <c r="H55" s="17"/>
+      <c r="I55" s="17"/>
+      <c r="J55" s="18">
+        <f>0.13*G53*(33.99)/10</f>
+        <v>22.53537</v>
+      </c>
+      <c r="K55" s="17"/>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A56" s="16"/>
+      <c r="B56" s="32" t="s">
+        <v>55</v>
+      </c>
+      <c r="C56" s="17"/>
+      <c r="D56" s="17"/>
+      <c r="E56" s="17"/>
+      <c r="F56" s="17"/>
+      <c r="G56" s="17"/>
+      <c r="H56" s="17"/>
+      <c r="I56" s="17"/>
+      <c r="J56" s="18">
+        <f>0.13*G53*(877.45/10)</f>
+        <v>581.74935000000005</v>
+      </c>
+      <c r="K56" s="17"/>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A57" s="16"/>
+      <c r="B57" s="17"/>
+      <c r="C57" s="17"/>
+      <c r="D57" s="17"/>
+      <c r="E57" s="17"/>
+      <c r="F57" s="17"/>
+      <c r="G57" s="17"/>
+      <c r="H57" s="17"/>
+      <c r="I57" s="17"/>
+      <c r="J57" s="17"/>
+      <c r="K57" s="17"/>
+    </row>
+    <row r="58" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="A58" s="16">
+        <v>7</v>
+      </c>
+      <c r="B58" s="37" t="s">
+        <v>56</v>
+      </c>
+      <c r="C58" s="17"/>
+      <c r="D58" s="17"/>
+      <c r="E58" s="17"/>
+      <c r="F58" s="17"/>
+      <c r="G58" s="17"/>
+      <c r="H58" s="17"/>
+      <c r="I58" s="17"/>
+      <c r="J58" s="17"/>
+      <c r="K58" s="17"/>
+    </row>
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A59" s="16"/>
+      <c r="B59" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="C59" s="17">
+        <v>1</v>
+      </c>
+      <c r="D59" s="33">
+        <f>D13</f>
+        <v>4</v>
+      </c>
+      <c r="E59" s="33">
+        <v>0.23</v>
+      </c>
+      <c r="F59" s="33">
+        <v>0.45</v>
+      </c>
+      <c r="G59" s="33">
+        <f>PRODUCT(C59:F59)</f>
+        <v>0.41400000000000003</v>
+      </c>
+      <c r="H59" s="17"/>
+      <c r="I59" s="17"/>
+      <c r="J59" s="17"/>
+      <c r="K59" s="17"/>
+      <c r="M59" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N59" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O59" s="33"/>
+      <c r="P59" s="33">
+        <f>PI()*M59*SQRT(M59^2+N59^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="60" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="2"/>
+      <c r="B60" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C60" s="3"/>
+      <c r="D60" s="4"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="5"/>
+      <c r="G60" s="6">
+        <f>SUM(G59:G59)</f>
+        <v>0.41400000000000003</v>
+      </c>
+      <c r="H60" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="I60" s="6">
+        <v>1754.28</v>
+      </c>
+      <c r="J60" s="18">
+        <f>G60*I60</f>
+        <v>726.27192000000002</v>
+      </c>
+      <c r="K60" s="5"/>
+    </row>
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A61" s="16"/>
+      <c r="B61" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="C61" s="17"/>
+      <c r="D61" s="17"/>
+      <c r="E61" s="17"/>
+      <c r="F61" s="17"/>
+      <c r="G61" s="17"/>
+      <c r="H61" s="17"/>
+      <c r="I61" s="17"/>
+      <c r="J61" s="18">
+        <f>0.13*G60*(8481.2)</f>
+        <v>456.45818400000007</v>
+      </c>
+      <c r="K61" s="17"/>
+    </row>
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A62" s="16"/>
+      <c r="B62" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="C62" s="17"/>
+      <c r="D62" s="17"/>
+      <c r="E62" s="17"/>
+      <c r="F62" s="17"/>
+      <c r="G62" s="17"/>
+      <c r="H62" s="17"/>
+      <c r="I62" s="17"/>
+      <c r="J62" s="18">
+        <f>0.13*G60*912.17</f>
+        <v>49.0929894</v>
+      </c>
+      <c r="K62" s="17"/>
+    </row>
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A63" s="16"/>
+      <c r="B63" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="C63" s="17"/>
+      <c r="D63" s="17"/>
+      <c r="E63" s="17"/>
+      <c r="F63" s="17"/>
+      <c r="G63" s="17"/>
+      <c r="H63" s="17"/>
+      <c r="I63" s="17"/>
+      <c r="J63" s="18">
+        <f>0.13*G60*953.37</f>
+        <v>51.310373400000003</v>
+      </c>
+      <c r="K63" s="17"/>
+    </row>
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A64" s="16"/>
+      <c r="B64" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="C64" s="17"/>
+      <c r="D64" s="17"/>
+      <c r="E64" s="17"/>
+      <c r="F64" s="17"/>
+      <c r="G64" s="17"/>
+      <c r="H64" s="17"/>
+      <c r="I64" s="17"/>
+      <c r="J64" s="18">
+        <f>0.13*G60*28</f>
+        <v>1.5069600000000003</v>
+      </c>
+      <c r="K64" s="17"/>
+    </row>
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A65" s="16"/>
+      <c r="B65" s="17"/>
+      <c r="C65" s="17"/>
+      <c r="D65" s="17"/>
+      <c r="E65" s="17"/>
+      <c r="F65" s="17"/>
+      <c r="G65" s="17"/>
+      <c r="H65" s="17"/>
+      <c r="I65" s="17"/>
+      <c r="J65" s="17"/>
+      <c r="K65" s="17"/>
+    </row>
+    <row r="66" spans="1:16" ht="150" x14ac:dyDescent="0.25">
+      <c r="A66" s="16">
+        <v>8</v>
+      </c>
+      <c r="B66" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="C66" s="17"/>
+      <c r="D66" s="17"/>
+      <c r="E66" s="17"/>
+      <c r="F66" s="17"/>
+      <c r="G66" s="17"/>
+      <c r="H66" s="17"/>
+      <c r="I66" s="17"/>
+      <c r="J66" s="17"/>
+      <c r="K66" s="17"/>
+    </row>
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A67" s="16"/>
+      <c r="B67" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="C67" s="17">
+        <v>1</v>
+      </c>
+      <c r="D67" s="33">
+        <v>15</v>
+      </c>
+      <c r="E67" s="33"/>
+      <c r="F67" s="33"/>
+      <c r="G67" s="33">
+        <f>PRODUCT(C67:F67)</f>
+        <v>15</v>
+      </c>
+      <c r="H67" s="17"/>
+      <c r="I67" s="17"/>
+      <c r="J67" s="17"/>
+      <c r="K67" s="17"/>
+      <c r="M67" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N67" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O67" s="33"/>
+      <c r="P67" s="33">
+        <f>PI()*M67*SQRT(M67^2+N67^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="68" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="2"/>
+      <c r="B68" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C68" s="3"/>
+      <c r="D68" s="4"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+      <c r="G68" s="6">
+        <f>SUM(G67:G67)</f>
+        <v>15</v>
+      </c>
+      <c r="H68" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="I68" s="6">
+        <v>4132.8</v>
+      </c>
+      <c r="J68" s="18">
+        <f>G68*I68</f>
+        <v>61992</v>
+      </c>
+      <c r="K68" s="5"/>
+    </row>
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A69" s="16"/>
+      <c r="B69" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="C69" s="17"/>
+      <c r="D69" s="17"/>
+      <c r="E69" s="17"/>
+      <c r="F69" s="17"/>
+      <c r="G69" s="17"/>
+      <c r="H69" s="17"/>
+      <c r="I69" s="17"/>
+      <c r="J69" s="18">
+        <f>0.13*J68</f>
+        <v>8058.96</v>
+      </c>
+      <c r="K69" s="17"/>
+    </row>
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A70" s="16"/>
+      <c r="B70" s="17"/>
+      <c r="C70" s="17"/>
+      <c r="D70" s="17"/>
+      <c r="E70" s="17"/>
+      <c r="F70" s="17"/>
+      <c r="G70" s="17"/>
+      <c r="H70" s="17"/>
+      <c r="I70" s="17"/>
+      <c r="J70" s="17"/>
+      <c r="K70" s="17"/>
+    </row>
+    <row r="71" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A71" s="16">
+        <v>9</v>
+      </c>
+      <c r="B71" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="C71" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D71" s="52" t="s">
+        <v>61</v>
+      </c>
+      <c r="E71" s="53" t="s">
+        <v>62</v>
+      </c>
+      <c r="F71" s="53" t="s">
+        <v>63</v>
+      </c>
+      <c r="G71" s="17"/>
+      <c r="H71" s="17"/>
+      <c r="I71" s="17"/>
+      <c r="J71" s="17"/>
+      <c r="K71" s="17"/>
+    </row>
+    <row r="72" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A72" s="16"/>
+      <c r="B72" s="54" t="s">
+        <v>64</v>
+      </c>
+      <c r="C72" s="17">
+        <v>1</v>
+      </c>
+      <c r="D72" s="33">
+        <f>4*(7.5/3.281)-(3/3.281)</f>
+        <v>8.2291984151173416</v>
+      </c>
+      <c r="E72" s="33">
+        <v>2.88</v>
+      </c>
+      <c r="F72" s="33">
+        <f>PRODUCT(C72:E72)</f>
+        <v>23.700091435537942</v>
+      </c>
+      <c r="G72" s="33">
+        <f>F72</f>
+        <v>23.700091435537942</v>
+      </c>
+      <c r="H72" s="17"/>
+      <c r="I72" s="17"/>
+      <c r="J72" s="17"/>
+      <c r="K72" s="17"/>
+      <c r="M72" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N72" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O72" s="33"/>
+      <c r="P72" s="33">
+        <f>PI()*M72*SQRT(M72^2+N72^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="73" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="A73" s="16"/>
+      <c r="B73" s="54" t="s">
+        <v>65</v>
+      </c>
+      <c r="C73" s="17">
+        <v>10</v>
+      </c>
+      <c r="D73" s="33">
+        <f>2.5/3.281</f>
+        <v>0.76196281621456874</v>
+      </c>
+      <c r="E73" s="33">
+        <v>3.54</v>
+      </c>
+      <c r="F73" s="33">
+        <f>PRODUCT(C73:E73)</f>
+        <v>26.973483693995735</v>
+      </c>
+      <c r="G73" s="33">
+        <f>F73</f>
+        <v>26.973483693995735</v>
+      </c>
+      <c r="H73" s="17"/>
+      <c r="I73" s="17"/>
+      <c r="J73" s="17"/>
+      <c r="K73" s="17"/>
+      <c r="M73" s="51"/>
+      <c r="N73" s="51"/>
+      <c r="O73" s="51"/>
+      <c r="P73" s="51"/>
+    </row>
+    <row r="74" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="2"/>
+      <c r="B74" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C74" s="3"/>
+      <c r="D74" s="4"/>
+      <c r="E74" s="5"/>
+      <c r="F74" s="5"/>
+      <c r="G74" s="6">
+        <f>SUM(G72:G73)</f>
+        <v>50.673575129533674</v>
+      </c>
+      <c r="H74" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="I74" s="6">
+        <v>182.51</v>
+      </c>
+      <c r="J74" s="18">
+        <f>G74*I74</f>
+        <v>9248.4341968911904</v>
+      </c>
+      <c r="K74" s="5"/>
+    </row>
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A75" s="16"/>
+      <c r="B75" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="C75" s="17"/>
+      <c r="D75" s="17"/>
+      <c r="E75" s="17"/>
+      <c r="F75" s="17"/>
+      <c r="G75" s="17"/>
+      <c r="H75" s="17"/>
+      <c r="I75" s="17"/>
+      <c r="J75" s="18">
+        <f>0.13*G74*(1871.42/18.94)</f>
+        <v>650.90287518260561</v>
+      </c>
+      <c r="K75" s="17"/>
+    </row>
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A76" s="16"/>
+      <c r="B76" s="17"/>
+      <c r="C76" s="17"/>
+      <c r="D76" s="17"/>
+      <c r="E76" s="17"/>
+      <c r="F76" s="17"/>
+      <c r="G76" s="17"/>
+      <c r="H76" s="17"/>
+      <c r="I76" s="17"/>
+      <c r="J76" s="17"/>
+      <c r="K76" s="17"/>
+    </row>
+    <row r="77" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="A77" s="2">
+        <v>10</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C77" s="3">
+        <v>1</v>
+      </c>
+      <c r="D77" s="4"/>
+      <c r="E77" s="5"/>
+      <c r="F77" s="5"/>
+      <c r="G77" s="7">
+        <f t="shared" ref="G77" si="7">PRODUCT(C77:F77)</f>
+        <v>1</v>
+      </c>
+      <c r="H77" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="I77" s="6">
+        <v>5000</v>
+      </c>
+      <c r="J77" s="7">
+        <f>G77*I77</f>
+        <v>5000</v>
+      </c>
+      <c r="K77" s="5"/>
+    </row>
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A78" s="2"/>
+      <c r="B78" s="8"/>
+      <c r="C78" s="3"/>
+      <c r="D78" s="4"/>
+      <c r="E78" s="5"/>
+      <c r="F78" s="5"/>
+      <c r="G78" s="6"/>
+      <c r="H78" s="7"/>
+      <c r="I78" s="6"/>
+      <c r="J78" s="18"/>
+      <c r="K78" s="5"/>
+    </row>
+    <row r="79" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="2">
+        <v>11</v>
+      </c>
+      <c r="B79" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C46" s="3">
+      <c r="C79" s="3">
         <v>1</v>
       </c>
-      <c r="D46" s="4"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="5"/>
-      <c r="G46" s="7">
-        <f t="shared" ref="G46" si="0">PRODUCT(C46:F46)</f>
+      <c r="D79" s="4"/>
+      <c r="E79" s="5"/>
+      <c r="F79" s="5"/>
+      <c r="G79" s="7">
+        <f t="shared" ref="G79" si="8">PRODUCT(C79:F79)</f>
         <v>1</v>
       </c>
-      <c r="H46" s="7" t="s">
+      <c r="H79" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="I46" s="6">
+      <c r="I79" s="6">
         <v>500</v>
       </c>
-      <c r="J46" s="7">
-        <f>G46*I46</f>
+      <c r="J79" s="7">
+        <f>G79*I79</f>
         <v>500</v>
       </c>
-      <c r="K46" s="5"/>
-    </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A47" s="2"/>
-      <c r="B47" s="8"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="5"/>
-      <c r="F47" s="5"/>
-      <c r="G47" s="6"/>
-      <c r="H47" s="7"/>
-      <c r="I47" s="6"/>
-      <c r="J47" s="18"/>
-      <c r="K47" s="5"/>
-    </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A48" s="21"/>
-      <c r="B48" s="22" t="s">
+      <c r="K79" s="5"/>
+    </row>
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A80" s="2"/>
+      <c r="B80" s="8"/>
+      <c r="C80" s="3"/>
+      <c r="D80" s="4"/>
+      <c r="E80" s="5"/>
+      <c r="F80" s="5"/>
+      <c r="G80" s="6"/>
+      <c r="H80" s="7"/>
+      <c r="I80" s="6"/>
+      <c r="J80" s="18"/>
+      <c r="K80" s="5"/>
+    </row>
+    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A81" s="21"/>
+      <c r="B81" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="C48" s="23"/>
-      <c r="D48" s="24"/>
-      <c r="E48" s="24"/>
-      <c r="F48" s="24"/>
-      <c r="G48" s="18"/>
-      <c r="H48" s="18"/>
-      <c r="I48" s="18"/>
-      <c r="J48" s="18">
-        <f>SUM(J9:J46)</f>
-        <v>506231.45545325003</v>
-      </c>
-      <c r="K48" s="25"/>
-    </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M49" s="20"/>
-      <c r="N49" s="20"/>
-      <c r="O49" s="20"/>
-      <c r="P49" s="20"/>
-      <c r="Q49" s="20"/>
-      <c r="R49" s="20"/>
-      <c r="S49" s="20"/>
-    </row>
-    <row r="50" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="26"/>
-      <c r="B50" s="27" t="s">
+      <c r="C81" s="23"/>
+      <c r="D81" s="24"/>
+      <c r="E81" s="24"/>
+      <c r="F81" s="24"/>
+      <c r="G81" s="18"/>
+      <c r="H81" s="18"/>
+      <c r="I81" s="18"/>
+      <c r="J81" s="18">
+        <f>SUM(J9:J79)</f>
+        <v>567007.79144636379</v>
+      </c>
+      <c r="K81" s="25"/>
+    </row>
+    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="M82" s="20"/>
+      <c r="N82" s="20"/>
+      <c r="O82" s="20"/>
+      <c r="P82" s="20"/>
+      <c r="Q82" s="20"/>
+      <c r="R82" s="20"/>
+      <c r="S82" s="20"/>
+    </row>
+    <row r="83" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="26"/>
+      <c r="B83" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C50" s="43">
-        <f>J48</f>
-        <v>506231.45545325003</v>
-      </c>
-      <c r="D50" s="44"/>
-      <c r="E50" s="9">
+      <c r="C83" s="38">
+        <f>J81</f>
+        <v>567007.79144636379</v>
+      </c>
+      <c r="D83" s="39"/>
+      <c r="E83" s="9">
         <v>100</v>
       </c>
-      <c r="F50" s="26"/>
-      <c r="G50" s="28"/>
-      <c r="H50" s="26"/>
-      <c r="I50" s="29"/>
-      <c r="J50" s="30"/>
-      <c r="K50" s="31"/>
-      <c r="M50" s="19"/>
-      <c r="N50" s="19"/>
-      <c r="O50" s="19"/>
-      <c r="P50" s="19"/>
-      <c r="Q50" s="19"/>
-      <c r="R50" s="19"/>
-      <c r="S50" s="19"/>
-    </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B51" s="27" t="s">
+      <c r="F83" s="26"/>
+      <c r="G83" s="28"/>
+      <c r="H83" s="26"/>
+      <c r="I83" s="29"/>
+      <c r="J83" s="30"/>
+      <c r="K83" s="31"/>
+      <c r="M83" s="19"/>
+      <c r="N83" s="19"/>
+      <c r="O83" s="19"/>
+      <c r="P83" s="19"/>
+      <c r="Q83" s="19"/>
+      <c r="R83" s="19"/>
+      <c r="S83" s="19"/>
+    </row>
+    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B84" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C51" s="47">
+      <c r="C84" s="42">
         <v>500000</v>
       </c>
-      <c r="D51" s="48"/>
-      <c r="E51" s="9"/>
-    </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B52" s="27" t="s">
+      <c r="D84" s="43"/>
+      <c r="E84" s="9"/>
+    </row>
+    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B85" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C52" s="47">
-        <f>C51-C54-C55</f>
+      <c r="C85" s="42">
+        <f>C84-C87-C88</f>
         <v>475000</v>
       </c>
-      <c r="D52" s="48"/>
-      <c r="E52" s="9">
-        <f>C52/C50*100</f>
-        <v>93.830597621539098</v>
-      </c>
-    </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B53" s="27" t="s">
+      <c r="D85" s="43"/>
+      <c r="E85" s="9">
+        <f>C85/C83*100</f>
+        <v>83.773099270529642</v>
+      </c>
+    </row>
+    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B86" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C53" s="49">
-        <f>C50-C52</f>
-        <v>31231.455453250033</v>
-      </c>
-      <c r="D53" s="49"/>
-      <c r="E53" s="9">
-        <f>100-E52</f>
-        <v>6.1694023784609016</v>
-      </c>
-    </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B54" s="27" t="s">
+      <c r="C86" s="44">
+        <f>C83-C85</f>
+        <v>92007.791446363786</v>
+      </c>
+      <c r="D86" s="44"/>
+      <c r="E86" s="9">
+        <f>100-E85</f>
+        <v>16.226900729470358</v>
+      </c>
+    </row>
+    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B87" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C54" s="43">
-        <f>C51*0.03</f>
+      <c r="C87" s="38">
+        <f>C84*0.03</f>
         <v>15000</v>
       </c>
-      <c r="D54" s="44"/>
-      <c r="E54" s="9">
+      <c r="D87" s="39"/>
+      <c r="E87" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B55" s="27" t="s">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B88" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="C55" s="43">
-        <f>C51*0.02</f>
+      <c r="C88" s="38">
+        <f>C84*0.02</f>
         <v>10000</v>
       </c>
-      <c r="D55" s="44"/>
-      <c r="E55" s="9">
+      <c r="D88" s="39"/>
+      <c r="E88" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="C54:D54"/>
-    <mergeCell ref="C55:D55"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="C50:D50"/>
-    <mergeCell ref="C51:D51"/>
-    <mergeCell ref="C52:D52"/>
-    <mergeCell ref="C53:D53"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="H6:K6"/>
     <mergeCell ref="A1:K1"/>
@@ -2172,6 +3102,14 @@
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A5:K5"/>
+    <mergeCell ref="C87:D87"/>
+    <mergeCell ref="C88:D88"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="C83:D83"/>
+    <mergeCell ref="C84:D84"/>
+    <mergeCell ref="C85:D85"/>
+    <mergeCell ref="C86:D86"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
@@ -2179,7 +3117,7 @@
     <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
   </headerFooter>
   <rowBreaks count="1" manualBreakCount="1">
-    <brk id="37" max="10" man="1"/>
+    <brk id="42" max="10" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
kalikamai mandir, jimbwal tol mandir truss, sangachok chaulagai tol mandir, bhotange chihanpaati estimate complete
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/नगर बजेट estimate/कालिकामाई मन्दिर पूर्वाधार विकास/कालिकामाई मन्दिर पूर्वाधार विकास.xlsx
+++ b/बजेट माग estimate/नगर बजेट estimate/कालिकामाई मन्दिर पूर्वाधार विकास/कालिकामाई मन्दिर पूर्वाधार विकास.xlsx
@@ -1,11 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D24A0467-1D26-4224-9028-2F0F9B370EEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="12" r:id="rId1"/>
@@ -278,10 +277,10 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -448,9 +447,9 @@
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
@@ -462,7 +461,7 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -486,14 +485,14 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -512,7 +511,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -527,7 +526,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -547,6 +546,34 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -566,42 +593,14 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Comma 2" xfId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Normal 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Percent 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 3" xfId="5"/>
+    <cellStyle name="Percent 2" xfId="4"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -617,7 +616,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -711,7 +710,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -770,11 +769,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Datasheet"/>
       <sheetName val="Abstract"/>
@@ -837,9 +833,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -877,9 +873,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -914,7 +910,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -949,7 +945,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1122,135 +1118,135 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:S88"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" style="19" customWidth="1"/>
-    <col min="2" max="2" width="30.85546875" style="19" customWidth="1"/>
-    <col min="3" max="3" width="4.42578125" style="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.42578125" style="19" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" style="19" customWidth="1"/>
-    <col min="6" max="6" width="7.28515625" style="19" customWidth="1"/>
-    <col min="7" max="7" width="9.140625" style="19"/>
+    <col min="1" max="1" width="4.6640625" style="19" customWidth="1"/>
+    <col min="2" max="2" width="30.88671875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.44140625" style="19" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" style="19" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" style="19" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" style="19"/>
     <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5703125" style="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="9.140625" style="19"/>
+    <col min="9" max="9" width="9.5546875" style="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="9.109375" style="19"/>
     <col min="13" max="16" width="0" style="19" hidden="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="19"/>
+    <col min="17" max="16384" width="9.109375" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="47" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
-      <c r="I1" s="47"/>
-      <c r="J1" s="47"/>
-      <c r="K1" s="47"/>
-    </row>
-    <row r="2" spans="1:16" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="48" t="s">
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+    </row>
+    <row r="2" spans="1:16" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="49" t="s">
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A3" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="49"/>
-      <c r="C3" s="49"/>
-      <c r="D3" s="49"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="49"/>
-      <c r="G3" s="49"/>
-      <c r="H3" s="49"/>
-      <c r="I3" s="49"/>
-      <c r="J3" s="49"/>
-      <c r="K3" s="49"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="49" t="s">
+      <c r="B3" s="46"/>
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
+      <c r="H3" s="46"/>
+      <c r="I3" s="46"/>
+      <c r="J3" s="46"/>
+      <c r="K3" s="46"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="49"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="49"/>
-      <c r="I4" s="49"/>
-      <c r="J4" s="49"/>
-      <c r="K4" s="49"/>
-    </row>
-    <row r="5" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="50" t="s">
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="46"/>
+      <c r="J4" s="46"/>
+      <c r="K4" s="46"/>
+    </row>
+    <row r="5" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A5" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="50"/>
-      <c r="C5" s="50"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="50"/>
-      <c r="G5" s="50"/>
-      <c r="H5" s="50"/>
-      <c r="I5" s="50"/>
-      <c r="J5" s="50"/>
-      <c r="K5" s="50"/>
-    </row>
-    <row r="6" spans="1:16" ht="18" x14ac:dyDescent="0.25">
-      <c r="A6" s="45" t="s">
+      <c r="B5" s="47"/>
+      <c r="C5" s="47"/>
+      <c r="D5" s="47"/>
+      <c r="E5" s="47"/>
+      <c r="F5" s="47"/>
+      <c r="G5" s="47"/>
+      <c r="H5" s="47"/>
+      <c r="I5" s="47"/>
+      <c r="J5" s="47"/>
+      <c r="K5" s="47"/>
+    </row>
+    <row r="6" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A6" s="42" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="45"/>
-      <c r="C6" s="45"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="42"/>
+      <c r="F6" s="42"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="46" t="s">
+      <c r="H6" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="46"/>
-      <c r="J6" s="46"/>
-      <c r="K6" s="46"/>
-    </row>
-    <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="40" t="s">
+      <c r="I6" s="43"/>
+      <c r="J6" s="43"/>
+      <c r="K6" s="43"/>
+    </row>
+    <row r="7" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="40"/>
-      <c r="C7" s="40"/>
-      <c r="D7" s="40"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="40"/>
+      <c r="B7" s="50"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="50"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="50"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="41" t="s">
+      <c r="H7" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="I7" s="41"/>
-      <c r="J7" s="41"/>
-      <c r="K7" s="41"/>
-    </row>
-    <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I7" s="51"/>
+      <c r="J7" s="51"/>
+      <c r="K7" s="51"/>
+    </row>
+    <row r="8" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
         <v>6</v>
       </c>
@@ -1285,7 +1281,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="180" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="171.6" x14ac:dyDescent="0.3">
       <c r="A9" s="16">
         <v>1</v>
       </c>
@@ -1302,7 +1298,7 @@
       <c r="J9" s="17"/>
       <c r="K9" s="17"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="16"/>
       <c r="B10" s="32" t="s">
         <v>47</v>
@@ -1341,7 +1337,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="16"/>
       <c r="B11" s="32"/>
       <c r="C11" s="17">
@@ -1365,12 +1361,12 @@
       <c r="I11" s="17"/>
       <c r="J11" s="17"/>
       <c r="K11" s="17"/>
-      <c r="M11" s="51"/>
-      <c r="N11" s="51"/>
-      <c r="O11" s="51"/>
-      <c r="P11" s="51"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M11" s="38"/>
+      <c r="N11" s="38"/>
+      <c r="O11" s="38"/>
+      <c r="P11" s="38"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="16"/>
       <c r="B12" s="32" t="s">
         <v>48</v>
@@ -1401,7 +1397,7 @@
       <c r="O12" s="36"/>
       <c r="P12" s="36"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="16"/>
       <c r="B13" s="32" t="s">
         <v>49</v>
@@ -1431,7 +1427,7 @@
       <c r="O13" s="36"/>
       <c r="P13" s="36"/>
     </row>
-    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="34" t="s">
         <v>17</v>
@@ -1456,7 +1452,7 @@
       </c>
       <c r="K14" s="5"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="16"/>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -1469,7 +1465,7 @@
       <c r="J15" s="17"/>
       <c r="K15" s="17"/>
     </row>
-    <row r="16" spans="1:16" ht="188.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A16" s="16">
         <v>2</v>
       </c>
@@ -1486,7 +1482,7 @@
       <c r="J16" s="17"/>
       <c r="K16" s="17"/>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="16"/>
       <c r="B17" s="32" t="s">
         <v>30</v>
@@ -1527,7 +1523,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="34" t="s">
         <v>17</v>
@@ -1552,7 +1548,7 @@
       </c>
       <c r="K18" s="5"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="16"/>
       <c r="B19" s="32" t="s">
         <v>24</v>
@@ -1570,7 +1566,7 @@
       </c>
       <c r="K19" s="17"/>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="16"/>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -1583,7 +1579,7 @@
       <c r="J20" s="17"/>
       <c r="K20" s="17"/>
     </row>
-    <row r="21" spans="1:16" ht="94.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="109.2" x14ac:dyDescent="0.3">
       <c r="A21" s="16">
         <v>3</v>
       </c>
@@ -1600,7 +1596,7 @@
       <c r="J21" s="17"/>
       <c r="K21" s="17"/>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="16"/>
       <c r="B22" s="32" t="str">
         <f>B17</f>
@@ -1642,7 +1638,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="16"/>
       <c r="B23" s="32" t="str">
         <f>B10</f>
@@ -1671,12 +1667,12 @@
       <c r="I23" s="17"/>
       <c r="J23" s="17"/>
       <c r="K23" s="17"/>
-      <c r="M23" s="51"/>
-      <c r="N23" s="51"/>
-      <c r="O23" s="51"/>
-      <c r="P23" s="51"/>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M23" s="38"/>
+      <c r="N23" s="38"/>
+      <c r="O23" s="38"/>
+      <c r="P23" s="38"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A24" s="16"/>
       <c r="B24" s="32"/>
       <c r="C24" s="17">
@@ -1702,12 +1698,12 @@
       <c r="I24" s="17"/>
       <c r="J24" s="17"/>
       <c r="K24" s="17"/>
-      <c r="M24" s="51"/>
-      <c r="N24" s="51"/>
-      <c r="O24" s="51"/>
-      <c r="P24" s="51"/>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="M24" s="38"/>
+      <c r="N24" s="38"/>
+      <c r="O24" s="38"/>
+      <c r="P24" s="38"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" s="16"/>
       <c r="B25" s="32" t="str">
         <f t="shared" ref="B25" si="3">B12</f>
@@ -1736,12 +1732,12 @@
       <c r="I25" s="17"/>
       <c r="J25" s="17"/>
       <c r="K25" s="17"/>
-      <c r="M25" s="51"/>
-      <c r="N25" s="51"/>
-      <c r="O25" s="51"/>
-      <c r="P25" s="51"/>
-    </row>
-    <row r="26" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M25" s="38"/>
+      <c r="N25" s="38"/>
+      <c r="O25" s="38"/>
+      <c r="P25" s="38"/>
+    </row>
+    <row r="26" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
       <c r="B26" s="34" t="s">
         <v>17</v>
@@ -1766,7 +1762,7 @@
       </c>
       <c r="K26" s="5"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" s="16"/>
       <c r="B27" s="32" t="s">
         <v>24</v>
@@ -1784,7 +1780,7 @@
       </c>
       <c r="K27" s="17"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" s="16"/>
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
@@ -1797,7 +1793,7 @@
       <c r="J28" s="17"/>
       <c r="K28" s="17"/>
     </row>
-    <row r="29" spans="1:16" ht="94.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A29" s="16">
         <v>4</v>
       </c>
@@ -1814,7 +1810,7 @@
       <c r="J29" s="17"/>
       <c r="K29" s="17"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" s="16"/>
       <c r="B30" s="32" t="str">
         <f>B22</f>
@@ -1856,7 +1852,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A31" s="16"/>
       <c r="B31" s="32"/>
       <c r="C31" s="17">
@@ -1885,7 +1881,7 @@
       <c r="O31" s="36"/>
       <c r="P31" s="36"/>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" s="16"/>
       <c r="B32" s="32" t="str">
         <f>B23</f>
@@ -1919,7 +1915,7 @@
       <c r="O32" s="36"/>
       <c r="P32" s="36"/>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A33" s="16"/>
       <c r="B33" s="32"/>
       <c r="C33" s="17">
@@ -1950,7 +1946,7 @@
       <c r="O33" s="36"/>
       <c r="P33" s="36"/>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A34" s="16"/>
       <c r="B34" s="32" t="str">
         <f>B25</f>
@@ -1984,7 +1980,7 @@
       <c r="O34" s="36"/>
       <c r="P34" s="36"/>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A35" s="16"/>
       <c r="B35" s="32" t="str">
         <f>B13</f>
@@ -2017,7 +2013,7 @@
       <c r="O35" s="36"/>
       <c r="P35" s="36"/>
     </row>
-    <row r="36" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
       <c r="B36" s="34" t="s">
         <v>17</v>
@@ -2042,7 +2038,7 @@
       </c>
       <c r="K36" s="5"/>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A37" s="16"/>
       <c r="B37" s="32" t="s">
         <v>33</v>
@@ -2060,7 +2056,7 @@
       </c>
       <c r="K37" s="17"/>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A38" s="16"/>
       <c r="B38" s="32" t="s">
         <v>34</v>
@@ -2078,7 +2074,7 @@
       </c>
       <c r="K38" s="17"/>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A39" s="16"/>
       <c r="B39" s="32" t="s">
         <v>35</v>
@@ -2096,7 +2092,7 @@
       </c>
       <c r="K39" s="17"/>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A40" s="16"/>
       <c r="B40" s="32" t="s">
         <v>36</v>
@@ -2114,7 +2110,7 @@
       </c>
       <c r="K40" s="17"/>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A41" s="16"/>
       <c r="B41" s="32" t="s">
         <v>40</v>
@@ -2132,7 +2128,7 @@
       </c>
       <c r="K41" s="17"/>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A42" s="16"/>
       <c r="B42" s="17"/>
       <c r="C42" s="17"/>
@@ -2145,7 +2141,7 @@
       <c r="J42" s="17"/>
       <c r="K42" s="17"/>
     </row>
-    <row r="43" spans="1:16" ht="110.25" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:16" ht="109.2" x14ac:dyDescent="0.3">
       <c r="A43" s="16">
         <v>5</v>
       </c>
@@ -2162,7 +2158,7 @@
       <c r="J43" s="17"/>
       <c r="K43" s="17"/>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A44" s="16"/>
       <c r="B44" s="32" t="str">
         <f>B30</f>
@@ -2204,7 +2200,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="45" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2"/>
       <c r="B45" s="34" t="s">
         <v>17</v>
@@ -2229,7 +2225,7 @@
       </c>
       <c r="K45" s="5"/>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A46" s="16"/>
       <c r="B46" s="32" t="s">
         <v>33</v>
@@ -2247,7 +2243,7 @@
       </c>
       <c r="K46" s="17"/>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A47" s="16"/>
       <c r="B47" s="32" t="s">
         <v>34</v>
@@ -2265,7 +2261,7 @@
       </c>
       <c r="K47" s="17"/>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A48" s="16"/>
       <c r="B48" s="32" t="s">
         <v>38</v>
@@ -2283,7 +2279,7 @@
       </c>
       <c r="K48" s="17"/>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A49" s="16"/>
       <c r="B49" s="32" t="s">
         <v>40</v>
@@ -2301,7 +2297,7 @@
       </c>
       <c r="K49" s="17"/>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A50" s="16"/>
       <c r="B50" s="17"/>
       <c r="C50" s="17"/>
@@ -2314,7 +2310,7 @@
       <c r="J50" s="17"/>
       <c r="K50" s="17"/>
     </row>
-    <row r="51" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16" ht="60" x14ac:dyDescent="0.3">
       <c r="A51" s="16">
         <v>6</v>
       </c>
@@ -2331,7 +2327,7 @@
       <c r="J51" s="17"/>
       <c r="K51" s="17"/>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A52" s="16"/>
       <c r="B52" s="32" t="s">
         <v>50</v>
@@ -2370,7 +2366,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="53" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
       <c r="B53" s="34" t="s">
         <v>17</v>
@@ -2395,7 +2391,7 @@
       </c>
       <c r="K53" s="5"/>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A54" s="16"/>
       <c r="B54" s="32" t="s">
         <v>53</v>
@@ -2413,7 +2409,7 @@
       </c>
       <c r="K54" s="17"/>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A55" s="16"/>
       <c r="B55" s="32" t="s">
         <v>54</v>
@@ -2431,7 +2427,7 @@
       </c>
       <c r="K55" s="17"/>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A56" s="16"/>
       <c r="B56" s="32" t="s">
         <v>55</v>
@@ -2449,7 +2445,7 @@
       </c>
       <c r="K56" s="17"/>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A57" s="16"/>
       <c r="B57" s="17"/>
       <c r="C57" s="17"/>
@@ -2462,7 +2458,7 @@
       <c r="J57" s="17"/>
       <c r="K57" s="17"/>
     </row>
-    <row r="58" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:16" ht="30" x14ac:dyDescent="0.3">
       <c r="A58" s="16">
         <v>7</v>
       </c>
@@ -2479,7 +2475,7 @@
       <c r="J58" s="17"/>
       <c r="K58" s="17"/>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A59" s="16"/>
       <c r="B59" s="32" t="s">
         <v>57</v>
@@ -2519,7 +2515,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="60" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2"/>
       <c r="B60" s="34" t="s">
         <v>17</v>
@@ -2544,7 +2540,7 @@
       </c>
       <c r="K60" s="5"/>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A61" s="16"/>
       <c r="B61" s="32" t="s">
         <v>59</v>
@@ -2562,7 +2558,7 @@
       </c>
       <c r="K61" s="17"/>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A62" s="16"/>
       <c r="B62" s="32" t="s">
         <v>33</v>
@@ -2580,7 +2576,7 @@
       </c>
       <c r="K62" s="17"/>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A63" s="16"/>
       <c r="B63" s="32" t="s">
         <v>34</v>
@@ -2598,7 +2594,7 @@
       </c>
       <c r="K63" s="17"/>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A64" s="16"/>
       <c r="B64" s="32" t="s">
         <v>40</v>
@@ -2616,7 +2612,7 @@
       </c>
       <c r="K64" s="17"/>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A65" s="16"/>
       <c r="B65" s="17"/>
       <c r="C65" s="17"/>
@@ -2629,7 +2625,7 @@
       <c r="J65" s="17"/>
       <c r="K65" s="17"/>
     </row>
-    <row r="66" spans="1:16" ht="150" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:16" ht="135" x14ac:dyDescent="0.3">
       <c r="A66" s="16">
         <v>8</v>
       </c>
@@ -2646,7 +2642,7 @@
       <c r="J66" s="17"/>
       <c r="K66" s="17"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A67" s="16"/>
       <c r="B67" s="32" t="s">
         <v>44</v>
@@ -2681,7 +2677,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="68" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2"/>
       <c r="B68" s="34" t="s">
         <v>17</v>
@@ -2706,7 +2702,7 @@
       </c>
       <c r="K68" s="5"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A69" s="16"/>
       <c r="B69" s="32" t="s">
         <v>24</v>
@@ -2724,7 +2720,7 @@
       </c>
       <c r="K69" s="17"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A70" s="16"/>
       <c r="B70" s="17"/>
       <c r="C70" s="17"/>
@@ -2737,7 +2733,7 @@
       <c r="J70" s="17"/>
       <c r="K70" s="17"/>
     </row>
-    <row r="71" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A71" s="16">
         <v>9</v>
       </c>
@@ -2747,13 +2743,13 @@
       <c r="C71" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="D71" s="52" t="s">
+      <c r="D71" s="39" t="s">
         <v>61</v>
       </c>
-      <c r="E71" s="53" t="s">
+      <c r="E71" s="40" t="s">
         <v>62</v>
       </c>
-      <c r="F71" s="53" t="s">
+      <c r="F71" s="40" t="s">
         <v>63</v>
       </c>
       <c r="G71" s="17"/>
@@ -2762,9 +2758,9 @@
       <c r="J71" s="17"/>
       <c r="K71" s="17"/>
     </row>
-    <row r="72" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A72" s="16"/>
-      <c r="B72" s="54" t="s">
+      <c r="B72" s="41" t="s">
         <v>64</v>
       </c>
       <c r="C72" s="17">
@@ -2803,9 +2799,9 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="73" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A73" s="16"/>
-      <c r="B73" s="54" t="s">
+      <c r="B73" s="41" t="s">
         <v>65</v>
       </c>
       <c r="C73" s="17">
@@ -2830,12 +2826,12 @@
       <c r="I73" s="17"/>
       <c r="J73" s="17"/>
       <c r="K73" s="17"/>
-      <c r="M73" s="51"/>
-      <c r="N73" s="51"/>
-      <c r="O73" s="51"/>
-      <c r="P73" s="51"/>
-    </row>
-    <row r="74" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M73" s="38"/>
+      <c r="N73" s="38"/>
+      <c r="O73" s="38"/>
+      <c r="P73" s="38"/>
+    </row>
+    <row r="74" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="2"/>
       <c r="B74" s="34" t="s">
         <v>17</v>
@@ -2860,7 +2856,7 @@
       </c>
       <c r="K74" s="5"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A75" s="16"/>
       <c r="B75" s="32" t="s">
         <v>24</v>
@@ -2878,7 +2874,7 @@
       </c>
       <c r="K75" s="17"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A76" s="16"/>
       <c r="B76" s="17"/>
       <c r="C76" s="17"/>
@@ -2891,7 +2887,7 @@
       <c r="J76" s="17"/>
       <c r="K76" s="17"/>
     </row>
-    <row r="77" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:16" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A77" s="2">
         <v>10</v>
       </c>
@@ -2920,7 +2916,7 @@
       </c>
       <c r="K77" s="5"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A78" s="2"/>
       <c r="B78" s="8"/>
       <c r="C78" s="3"/>
@@ -2933,7 +2929,7 @@
       <c r="J78" s="18"/>
       <c r="K78" s="5"/>
     </row>
-    <row r="79" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
         <v>11</v>
       </c>
@@ -2962,7 +2958,7 @@
       </c>
       <c r="K79" s="5"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A80" s="2"/>
       <c r="B80" s="8"/>
       <c r="C80" s="3"/>
@@ -2975,7 +2971,7 @@
       <c r="J80" s="18"/>
       <c r="K80" s="5"/>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A81" s="21"/>
       <c r="B81" s="22" t="s">
         <v>22</v>
@@ -2993,7 +2989,7 @@
       </c>
       <c r="K81" s="25"/>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.3">
       <c r="M82" s="20"/>
       <c r="N82" s="20"/>
       <c r="O82" s="20"/>
@@ -3002,16 +2998,16 @@
       <c r="R82" s="20"/>
       <c r="S82" s="20"/>
     </row>
-    <row r="83" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A83" s="26"/>
       <c r="B83" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C83" s="38">
+      <c r="C83" s="48">
         <f>J81</f>
         <v>567007.79144636379</v>
       </c>
-      <c r="D83" s="39"/>
+      <c r="D83" s="49"/>
       <c r="E83" s="9">
         <v>100</v>
       </c>
@@ -3029,79 +3025,72 @@
       <c r="R83" s="19"/>
       <c r="S83" s="19"/>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B84" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C84" s="42">
+      <c r="C84" s="52">
         <v>500000</v>
       </c>
-      <c r="D84" s="43"/>
+      <c r="D84" s="53"/>
       <c r="E84" s="9"/>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B85" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C85" s="42">
+      <c r="C85" s="52">
         <f>C84-C87-C88</f>
         <v>475000</v>
       </c>
-      <c r="D85" s="43"/>
+      <c r="D85" s="53"/>
       <c r="E85" s="9">
         <f>C85/C83*100</f>
         <v>83.773099270529642</v>
       </c>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B86" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C86" s="44">
+      <c r="C86" s="54">
         <f>C83-C85</f>
         <v>92007.791446363786</v>
       </c>
-      <c r="D86" s="44"/>
+      <c r="D86" s="54"/>
       <c r="E86" s="9">
         <f>100-E85</f>
         <v>16.226900729470358</v>
       </c>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B87" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C87" s="38">
+      <c r="C87" s="48">
         <f>C84*0.03</f>
         <v>15000</v>
       </c>
-      <c r="D87" s="39"/>
+      <c r="D87" s="49"/>
       <c r="E87" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B88" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="C88" s="38">
+      <c r="C88" s="48">
         <f>C84*0.02</f>
         <v>10000</v>
       </c>
-      <c r="D88" s="39"/>
+      <c r="D88" s="49"/>
       <c r="E88" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C87:D87"/>
     <mergeCell ref="C88:D88"/>
     <mergeCell ref="A7:F7"/>
@@ -3110,6 +3099,13 @@
     <mergeCell ref="C84:D84"/>
     <mergeCell ref="C85:D85"/>
     <mergeCell ref="C86:D86"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>

</xml_diff>

<commit_message>
estimates detail given to ward head
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/नगर बजेट estimate/कालिकामाई मन्दिर पूर्वाधार विकास/कालिकामाई मन्दिर पूर्वाधार विकास.xlsx
+++ b/बजेट माग estimate/नगर बजेट estimate/कालिकामाई मन्दिर पूर्वाधार विकास/कालिकामाई मन्दिर पूर्वाधार विकास.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED2711EE-9B9C-4A5F-A720-E76B084DECC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="12" r:id="rId1"/>
@@ -72,9 +73,6 @@
     <t>Detail Estimated Sheet</t>
   </si>
   <si>
-    <t>Location:- Shankharapur Municipality 9</t>
-  </si>
-  <si>
     <t>S.N.</t>
   </si>
   <si>
@@ -273,14 +271,17 @@
   <si>
     <t>PS</t>
   </si>
+  <si>
+    <t>Location:- Shankharapur Municipality 1</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -447,13 +448,13 @@
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -461,7 +462,7 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -485,14 +486,14 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -511,7 +512,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -526,7 +527,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -546,7 +547,6 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -555,24 +555,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -593,14 +575,32 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="3"/>
+    <cellStyle name="Comma 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2"/>
-    <cellStyle name="Normal 3" xfId="5"/>
-    <cellStyle name="Percent 2" xfId="4"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Normal 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Percent 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -616,7 +616,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -710,7 +710,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -769,7 +769,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -833,9 +833,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -873,9 +873,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -910,7 +910,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -945,7 +945,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1118,175 +1118,175 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S88"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" style="19" customWidth="1"/>
-    <col min="2" max="2" width="30.88671875" style="19" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" style="19" customWidth="1"/>
-    <col min="5" max="5" width="8.5546875" style="19" customWidth="1"/>
-    <col min="6" max="6" width="7.33203125" style="19" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="19"/>
+    <col min="1" max="1" width="4.7109375" style="19" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" style="19" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" style="19" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" style="19" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="19"/>
     <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5546875" style="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.6640625" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="9.109375" style="19"/>
-    <col min="13" max="16" width="0" style="19" hidden="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.109375" style="19"/>
+    <col min="9" max="9" width="9.5703125" style="19" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="19" customWidth="1"/>
+    <col min="11" max="12" width="9.140625" style="19"/>
+    <col min="13" max="16" width="9.140625" style="19" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A1" s="44" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-    </row>
-    <row r="2" spans="1:16" ht="22.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="45" t="s">
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+    </row>
+    <row r="2" spans="1:16" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="51" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A3" s="46" t="s">
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="I2" s="51"/>
+      <c r="J2" s="51"/>
+      <c r="K2" s="51"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A4" s="46" t="s">
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="52"/>
+      <c r="E3" s="52"/>
+      <c r="F3" s="52"/>
+      <c r="G3" s="52"/>
+      <c r="H3" s="52"/>
+      <c r="I3" s="52"/>
+      <c r="J3" s="52"/>
+      <c r="K3" s="52"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46"/>
-      <c r="I4" s="46"/>
-      <c r="J4" s="46"/>
-      <c r="K4" s="46"/>
-    </row>
-    <row r="5" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A5" s="47" t="s">
+      <c r="B4" s="52"/>
+      <c r="C4" s="52"/>
+      <c r="D4" s="52"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="52"/>
+      <c r="G4" s="52"/>
+      <c r="H4" s="52"/>
+      <c r="I4" s="52"/>
+      <c r="J4" s="52"/>
+      <c r="K4" s="52"/>
+    </row>
+    <row r="5" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="47"/>
-      <c r="C5" s="47"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
-      <c r="F5" s="47"/>
-      <c r="G5" s="47"/>
-      <c r="H5" s="47"/>
-      <c r="I5" s="47"/>
-      <c r="J5" s="47"/>
-      <c r="K5" s="47"/>
-    </row>
-    <row r="6" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A6" s="42" t="s">
-        <v>43</v>
-      </c>
-      <c r="B6" s="42"/>
-      <c r="C6" s="42"/>
-      <c r="D6" s="42"/>
-      <c r="E6" s="42"/>
-      <c r="F6" s="42"/>
+      <c r="B5" s="53"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="53"/>
+      <c r="E5" s="53"/>
+      <c r="F5" s="53"/>
+      <c r="G5" s="53"/>
+      <c r="H5" s="53"/>
+      <c r="I5" s="53"/>
+      <c r="J5" s="53"/>
+      <c r="K5" s="53"/>
+    </row>
+    <row r="6" spans="1:16" ht="18" x14ac:dyDescent="0.25">
+      <c r="A6" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="48"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="43" t="s">
-        <v>29</v>
-      </c>
-      <c r="I6" s="43"/>
-      <c r="J6" s="43"/>
-      <c r="K6" s="43"/>
-    </row>
-    <row r="7" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="50" t="s">
+      <c r="H6" s="49" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="49"/>
+      <c r="J6" s="49"/>
+      <c r="K6" s="49"/>
+    </row>
+    <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="43" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="43"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="44" t="s">
+        <v>22</v>
+      </c>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="44"/>
+    </row>
+    <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="50"/>
-      <c r="C7" s="50"/>
-      <c r="D7" s="50"/>
-      <c r="E7" s="50"/>
-      <c r="F7" s="50"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="51" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" s="51"/>
-      <c r="J7" s="51"/>
-      <c r="K7" s="51"/>
-    </row>
-    <row r="8" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="12" t="s">
+      <c r="B8" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="C8" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="D8" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="E8" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="F8" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="G8" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="H8" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="I8" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="I8" s="14" t="s">
+      <c r="J8" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="14" t="s">
+      <c r="K8" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="K8" s="15" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" ht="171.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:16" ht="157.5" x14ac:dyDescent="0.25">
       <c r="A9" s="16">
         <v>1</v>
       </c>
       <c r="B9" s="35" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C9" s="17"/>
       <c r="D9" s="17"/>
@@ -1298,10 +1298,10 @@
       <c r="J9" s="17"/>
       <c r="K9" s="17"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="32" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C10" s="17">
         <v>1</v>
@@ -1337,7 +1337,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
       <c r="B11" s="32"/>
       <c r="C11" s="17">
@@ -1361,15 +1361,15 @@
       <c r="I11" s="17"/>
       <c r="J11" s="17"/>
       <c r="K11" s="17"/>
-      <c r="M11" s="38"/>
-      <c r="N11" s="38"/>
-      <c r="O11" s="38"/>
-      <c r="P11" s="38"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M11" s="36"/>
+      <c r="N11" s="36"/>
+      <c r="O11" s="36"/>
+      <c r="P11" s="36"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
       <c r="B12" s="32" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C12" s="17">
         <v>1</v>
@@ -1397,10 +1397,10 @@
       <c r="O12" s="36"/>
       <c r="P12" s="36"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
       <c r="B13" s="32" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C13" s="17">
         <v>1</v>
@@ -1427,10 +1427,10 @@
       <c r="O13" s="36"/>
       <c r="P13" s="36"/>
     </row>
-    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="4"/>
@@ -1441,7 +1441,7 @@
         <v>9.9652264553489776</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I14" s="6">
         <v>748.9</v>
@@ -1452,7 +1452,7 @@
       </c>
       <c r="K14" s="5"/>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -1465,12 +1465,12 @@
       <c r="J15" s="17"/>
       <c r="K15" s="17"/>
     </row>
-    <row r="16" spans="1:16" ht="187.2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="173.25" x14ac:dyDescent="0.25">
       <c r="A16" s="16">
         <v>2</v>
       </c>
       <c r="B16" s="35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C16" s="17"/>
       <c r="D16" s="17"/>
@@ -1482,10 +1482,10 @@
       <c r="J16" s="17"/>
       <c r="K16" s="17"/>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="16"/>
       <c r="B17" s="32" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C17" s="17">
         <v>1</v>
@@ -1523,10 +1523,10 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="4"/>
@@ -1537,7 +1537,7 @@
         <v>8.8006705272782693</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I18" s="6">
         <v>62.95</v>
@@ -1548,10 +1548,10 @@
       </c>
       <c r="K18" s="5"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="16"/>
       <c r="B19" s="32" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C19" s="17"/>
       <c r="D19" s="17"/>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="K19" s="17"/>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="16"/>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -1579,12 +1579,12 @@
       <c r="J20" s="17"/>
       <c r="K20" s="17"/>
     </row>
-    <row r="21" spans="1:16" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:16" ht="110.25" x14ac:dyDescent="0.25">
       <c r="A21" s="16">
         <v>3</v>
       </c>
       <c r="B21" s="35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C21" s="17"/>
       <c r="D21" s="17"/>
@@ -1596,7 +1596,7 @@
       <c r="J21" s="17"/>
       <c r="K21" s="17"/>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="16"/>
       <c r="B22" s="32" t="str">
         <f>B17</f>
@@ -1638,7 +1638,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="16"/>
       <c r="B23" s="32" t="str">
         <f>B10</f>
@@ -1667,12 +1667,12 @@
       <c r="I23" s="17"/>
       <c r="J23" s="17"/>
       <c r="K23" s="17"/>
-      <c r="M23" s="38"/>
-      <c r="N23" s="38"/>
-      <c r="O23" s="38"/>
-      <c r="P23" s="38"/>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M23" s="36"/>
+      <c r="N23" s="36"/>
+      <c r="O23" s="36"/>
+      <c r="P23" s="36"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="16"/>
       <c r="B24" s="32"/>
       <c r="C24" s="17">
@@ -1698,12 +1698,12 @@
       <c r="I24" s="17"/>
       <c r="J24" s="17"/>
       <c r="K24" s="17"/>
-      <c r="M24" s="38"/>
-      <c r="N24" s="38"/>
-      <c r="O24" s="38"/>
-      <c r="P24" s="38"/>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="M24" s="36"/>
+      <c r="N24" s="36"/>
+      <c r="O24" s="36"/>
+      <c r="P24" s="36"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="16"/>
       <c r="B25" s="32" t="str">
         <f t="shared" ref="B25" si="3">B12</f>
@@ -1732,15 +1732,15 @@
       <c r="I25" s="17"/>
       <c r="J25" s="17"/>
       <c r="K25" s="17"/>
-      <c r="M25" s="38"/>
-      <c r="N25" s="38"/>
-      <c r="O25" s="38"/>
-      <c r="P25" s="38"/>
-    </row>
-    <row r="26" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M25" s="36"/>
+      <c r="N25" s="36"/>
+      <c r="O25" s="36"/>
+      <c r="P25" s="36"/>
+    </row>
+    <row r="26" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C26" s="3"/>
       <c r="D26" s="4"/>
@@ -1751,7 +1751,7 @@
         <v>11.587360560804632</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I26" s="6">
         <v>4458.5200000000004</v>
@@ -1762,10 +1762,10 @@
       </c>
       <c r="K26" s="5"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" s="16"/>
       <c r="B27" s="32" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
@@ -1780,7 +1780,7 @@
       </c>
       <c r="K27" s="17"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" s="16"/>
       <c r="B28" s="17"/>
       <c r="C28" s="17"/>
@@ -1793,12 +1793,12 @@
       <c r="J28" s="17"/>
       <c r="K28" s="17"/>
     </row>
-    <row r="29" spans="1:16" ht="93.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:16" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A29" s="16">
         <v>4</v>
       </c>
       <c r="B29" s="35" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C29" s="17"/>
       <c r="D29" s="17"/>
@@ -1810,7 +1810,7 @@
       <c r="J29" s="17"/>
       <c r="K29" s="17"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
       <c r="B30" s="32" t="str">
         <f>B22</f>
@@ -1852,7 +1852,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="16"/>
       <c r="B31" s="32"/>
       <c r="C31" s="17">
@@ -1881,7 +1881,7 @@
       <c r="O31" s="36"/>
       <c r="P31" s="36"/>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="16"/>
       <c r="B32" s="32" t="str">
         <f>B23</f>
@@ -1915,7 +1915,7 @@
       <c r="O32" s="36"/>
       <c r="P32" s="36"/>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" s="16"/>
       <c r="B33" s="32"/>
       <c r="C33" s="17">
@@ -1946,7 +1946,7 @@
       <c r="O33" s="36"/>
       <c r="P33" s="36"/>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" s="16"/>
       <c r="B34" s="32" t="str">
         <f>B25</f>
@@ -1980,7 +1980,7 @@
       <c r="O34" s="36"/>
       <c r="P34" s="36"/>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" s="16"/>
       <c r="B35" s="32" t="str">
         <f>B13</f>
@@ -2013,10 +2013,10 @@
       <c r="O35" s="36"/>
       <c r="P35" s="36"/>
     </row>
-    <row r="36" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="4"/>
@@ -2027,7 +2027,7 @@
         <v>4.2734779030783301</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I36" s="6">
         <v>10964.46</v>
@@ -2038,10 +2038,10 @@
       </c>
       <c r="K36" s="5"/>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" s="16"/>
       <c r="B37" s="32" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C37" s="17"/>
       <c r="D37" s="17"/>
@@ -2056,10 +2056,10 @@
       </c>
       <c r="K37" s="17"/>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" s="16"/>
       <c r="B38" s="32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C38" s="17"/>
       <c r="D38" s="17"/>
@@ -2074,10 +2074,10 @@
       </c>
       <c r="K38" s="17"/>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" s="16"/>
       <c r="B39" s="32" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C39" s="17"/>
       <c r="D39" s="17"/>
@@ -2092,10 +2092,10 @@
       </c>
       <c r="K39" s="17"/>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" s="16"/>
       <c r="B40" s="32" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C40" s="17"/>
       <c r="D40" s="17"/>
@@ -2110,10 +2110,10 @@
       </c>
       <c r="K40" s="17"/>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" s="16"/>
       <c r="B41" s="32" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C41" s="17"/>
       <c r="D41" s="17"/>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="K41" s="17"/>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" s="16"/>
       <c r="B42" s="17"/>
       <c r="C42" s="17"/>
@@ -2141,12 +2141,12 @@
       <c r="J42" s="17"/>
       <c r="K42" s="17"/>
     </row>
-    <row r="43" spans="1:16" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" ht="110.25" x14ac:dyDescent="0.25">
       <c r="A43" s="16">
         <v>5</v>
       </c>
       <c r="B43" s="35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C43" s="17"/>
       <c r="D43" s="17"/>
@@ -2158,7 +2158,7 @@
       <c r="J43" s="17"/>
       <c r="K43" s="17"/>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" s="16"/>
       <c r="B44" s="32" t="str">
         <f>B30</f>
@@ -2200,10 +2200,10 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="45" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2"/>
       <c r="B45" s="34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C45" s="3"/>
       <c r="D45" s="4"/>
@@ -2214,7 +2214,7 @@
         <v>27.868790003047852</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I45" s="6">
         <v>8987.83</v>
@@ -2225,10 +2225,10 @@
       </c>
       <c r="K45" s="5"/>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A46" s="16"/>
       <c r="B46" s="32" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C46" s="17"/>
       <c r="D46" s="17"/>
@@ -2243,10 +2243,10 @@
       </c>
       <c r="K46" s="17"/>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A47" s="16"/>
       <c r="B47" s="32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C47" s="17"/>
       <c r="D47" s="17"/>
@@ -2261,10 +2261,10 @@
       </c>
       <c r="K47" s="17"/>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A48" s="16"/>
       <c r="B48" s="32" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C48" s="17"/>
       <c r="D48" s="17"/>
@@ -2279,10 +2279,10 @@
       </c>
       <c r="K48" s="17"/>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" s="16"/>
       <c r="B49" s="32" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C49" s="17"/>
       <c r="D49" s="17"/>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="K49" s="17"/>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" s="16"/>
       <c r="B50" s="17"/>
       <c r="C50" s="17"/>
@@ -2310,12 +2310,12 @@
       <c r="J50" s="17"/>
       <c r="K50" s="17"/>
     </row>
-    <row r="51" spans="1:16" ht="60" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A51" s="16">
         <v>6</v>
       </c>
       <c r="B51" s="37" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C51" s="17"/>
       <c r="D51" s="17"/>
@@ -2327,10 +2327,10 @@
       <c r="J51" s="17"/>
       <c r="K51" s="17"/>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" s="16"/>
       <c r="B52" s="32" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C52" s="17">
         <v>1</v>
@@ -2366,10 +2366,10 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="53" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
       <c r="B53" s="34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="4"/>
@@ -2380,7 +2380,7 @@
         <v>51</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I53" s="6">
         <v>1754.28</v>
@@ -2391,10 +2391,10 @@
       </c>
       <c r="K53" s="5"/>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" s="16"/>
       <c r="B54" s="32" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C54" s="17"/>
       <c r="D54" s="17"/>
@@ -2409,10 +2409,10 @@
       </c>
       <c r="K54" s="17"/>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" s="16"/>
       <c r="B55" s="32" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C55" s="17"/>
       <c r="D55" s="17"/>
@@ -2427,10 +2427,10 @@
       </c>
       <c r="K55" s="17"/>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A56" s="16"/>
       <c r="B56" s="32" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C56" s="17"/>
       <c r="D56" s="17"/>
@@ -2445,7 +2445,7 @@
       </c>
       <c r="K56" s="17"/>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A57" s="16"/>
       <c r="B57" s="17"/>
       <c r="C57" s="17"/>
@@ -2458,12 +2458,12 @@
       <c r="J57" s="17"/>
       <c r="K57" s="17"/>
     </row>
-    <row r="58" spans="1:16" ht="30" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="16">
         <v>7</v>
       </c>
       <c r="B58" s="37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C58" s="17"/>
       <c r="D58" s="17"/>
@@ -2475,10 +2475,10 @@
       <c r="J58" s="17"/>
       <c r="K58" s="17"/>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A59" s="16"/>
       <c r="B59" s="32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C59" s="17">
         <v>1</v>
@@ -2515,10 +2515,10 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="60" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2"/>
       <c r="B60" s="34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C60" s="3"/>
       <c r="D60" s="4"/>
@@ -2529,7 +2529,7 @@
         <v>0.41400000000000003</v>
       </c>
       <c r="H60" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I60" s="6">
         <v>1754.28</v>
@@ -2540,10 +2540,10 @@
       </c>
       <c r="K60" s="5"/>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A61" s="16"/>
       <c r="B61" s="32" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C61" s="17"/>
       <c r="D61" s="17"/>
@@ -2558,10 +2558,10 @@
       </c>
       <c r="K61" s="17"/>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A62" s="16"/>
       <c r="B62" s="32" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C62" s="17"/>
       <c r="D62" s="17"/>
@@ -2576,10 +2576,10 @@
       </c>
       <c r="K62" s="17"/>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A63" s="16"/>
       <c r="B63" s="32" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C63" s="17"/>
       <c r="D63" s="17"/>
@@ -2594,10 +2594,10 @@
       </c>
       <c r="K63" s="17"/>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" s="16"/>
       <c r="B64" s="32" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C64" s="17"/>
       <c r="D64" s="17"/>
@@ -2612,7 +2612,7 @@
       </c>
       <c r="K64" s="17"/>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="16"/>
       <c r="B65" s="17"/>
       <c r="C65" s="17"/>
@@ -2625,12 +2625,12 @@
       <c r="J65" s="17"/>
       <c r="K65" s="17"/>
     </row>
-    <row r="66" spans="1:16" ht="135" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:16" ht="150" x14ac:dyDescent="0.25">
       <c r="A66" s="16">
         <v>8</v>
       </c>
       <c r="B66" s="37" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C66" s="17"/>
       <c r="D66" s="17"/>
@@ -2642,10 +2642,10 @@
       <c r="J66" s="17"/>
       <c r="K66" s="17"/>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A67" s="16"/>
       <c r="B67" s="32" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C67" s="17">
         <v>1</v>
@@ -2677,10 +2677,10 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="68" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2"/>
       <c r="B68" s="34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C68" s="3"/>
       <c r="D68" s="4"/>
@@ -2691,7 +2691,7 @@
         <v>15</v>
       </c>
       <c r="H68" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I68" s="6">
         <v>4132.8</v>
@@ -2702,10 +2702,10 @@
       </c>
       <c r="K68" s="5"/>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A69" s="16"/>
       <c r="B69" s="32" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C69" s="17"/>
       <c r="D69" s="17"/>
@@ -2720,7 +2720,7 @@
       </c>
       <c r="K69" s="17"/>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A70" s="16"/>
       <c r="B70" s="17"/>
       <c r="C70" s="17"/>
@@ -2733,24 +2733,24 @@
       <c r="J70" s="17"/>
       <c r="K70" s="17"/>
     </row>
-    <row r="71" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A71" s="16">
         <v>9</v>
       </c>
       <c r="B71" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="C71" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="D71" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="C71" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="D71" s="39" t="s">
+      <c r="E71" s="39" t="s">
         <v>61</v>
       </c>
-      <c r="E71" s="40" t="s">
+      <c r="F71" s="39" t="s">
         <v>62</v>
-      </c>
-      <c r="F71" s="40" t="s">
-        <v>63</v>
       </c>
       <c r="G71" s="17"/>
       <c r="H71" s="17"/>
@@ -2758,10 +2758,10 @@
       <c r="J71" s="17"/>
       <c r="K71" s="17"/>
     </row>
-    <row r="72" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A72" s="16"/>
-      <c r="B72" s="41" t="s">
-        <v>64</v>
+      <c r="B72" s="40" t="s">
+        <v>63</v>
       </c>
       <c r="C72" s="17">
         <v>1</v>
@@ -2799,10 +2799,10 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="73" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A73" s="16"/>
-      <c r="B73" s="41" t="s">
-        <v>65</v>
+      <c r="B73" s="40" t="s">
+        <v>64</v>
       </c>
       <c r="C73" s="17">
         <v>10</v>
@@ -2826,15 +2826,15 @@
       <c r="I73" s="17"/>
       <c r="J73" s="17"/>
       <c r="K73" s="17"/>
-      <c r="M73" s="38"/>
-      <c r="N73" s="38"/>
-      <c r="O73" s="38"/>
-      <c r="P73" s="38"/>
-    </row>
-    <row r="74" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="M73" s="36"/>
+      <c r="N73" s="36"/>
+      <c r="O73" s="36"/>
+      <c r="P73" s="36"/>
+    </row>
+    <row r="74" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2"/>
       <c r="B74" s="34" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C74" s="3"/>
       <c r="D74" s="4"/>
@@ -2845,7 +2845,7 @@
         <v>50.673575129533674</v>
       </c>
       <c r="H74" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I74" s="6">
         <v>182.51</v>
@@ -2856,10 +2856,10 @@
       </c>
       <c r="K74" s="5"/>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A75" s="16"/>
       <c r="B75" s="32" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C75" s="17"/>
       <c r="D75" s="17"/>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="K75" s="17"/>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A76" s="16"/>
       <c r="B76" s="17"/>
       <c r="C76" s="17"/>
@@ -2887,12 +2887,12 @@
       <c r="J76" s="17"/>
       <c r="K76" s="17"/>
     </row>
-    <row r="77" spans="1:16" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
         <v>10</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C77" s="3">
         <v>1</v>
@@ -2905,18 +2905,18 @@
         <v>1</v>
       </c>
       <c r="H77" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I77" s="6">
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="J77" s="7">
         <f>G77*I77</f>
-        <v>5000</v>
+        <v>7000</v>
       </c>
       <c r="K77" s="5"/>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A78" s="2"/>
       <c r="B78" s="8"/>
       <c r="C78" s="3"/>
@@ -2929,12 +2929,12 @@
       <c r="J78" s="18"/>
       <c r="K78" s="5"/>
     </row>
-    <row r="79" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
         <v>11</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C79" s="3">
         <v>1</v>
@@ -2947,7 +2947,7 @@
         <v>1</v>
       </c>
       <c r="H79" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I79" s="6">
         <v>500</v>
@@ -2958,7 +2958,7 @@
       </c>
       <c r="K79" s="5"/>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A80" s="2"/>
       <c r="B80" s="8"/>
       <c r="C80" s="3"/>
@@ -2971,10 +2971,10 @@
       <c r="J80" s="18"/>
       <c r="K80" s="5"/>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A81" s="21"/>
       <c r="B81" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C81" s="23"/>
       <c r="D81" s="24"/>
@@ -2984,12 +2984,12 @@
       <c r="H81" s="18"/>
       <c r="I81" s="18"/>
       <c r="J81" s="18">
-        <f>SUM(J9:J79)</f>
-        <v>567007.79144636379</v>
+        <f>SUM(J10:J79)</f>
+        <v>569007.79144636379</v>
       </c>
       <c r="K81" s="25"/>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
       <c r="M82" s="20"/>
       <c r="N82" s="20"/>
       <c r="O82" s="20"/>
@@ -2998,16 +2998,16 @@
       <c r="R82" s="20"/>
       <c r="S82" s="20"/>
     </row>
-    <row r="83" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="26"/>
       <c r="B83" s="27" t="s">
-        <v>21</v>
-      </c>
-      <c r="C83" s="48">
+        <v>20</v>
+      </c>
+      <c r="C83" s="41">
         <f>J81</f>
-        <v>567007.79144636379</v>
-      </c>
-      <c r="D83" s="49"/>
+        <v>569007.79144636379</v>
+      </c>
+      <c r="D83" s="42"/>
       <c r="E83" s="9">
         <v>100</v>
       </c>
@@ -3025,72 +3025,79 @@
       <c r="R83" s="19"/>
       <c r="S83" s="19"/>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B84" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="C84" s="45">
+        <v>500000</v>
+      </c>
+      <c r="D84" s="46"/>
+      <c r="E84" s="9"/>
+    </row>
+    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B85" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C84" s="52">
-        <v>500000</v>
-      </c>
-      <c r="D84" s="53"/>
-      <c r="E84" s="9"/>
-    </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="B85" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="C85" s="52">
+      <c r="C85" s="45">
         <f>C84-C87-C88</f>
         <v>475000</v>
       </c>
-      <c r="D85" s="53"/>
+      <c r="D85" s="46"/>
       <c r="E85" s="9">
         <f>C85/C83*100</f>
-        <v>83.773099270529642</v>
-      </c>
-    </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.3">
+        <v>83.47864601161173</v>
+      </c>
+    </row>
+    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B86" s="27" t="s">
-        <v>41</v>
-      </c>
-      <c r="C86" s="54">
+        <v>40</v>
+      </c>
+      <c r="C86" s="47">
         <f>C83-C85</f>
-        <v>92007.791446363786</v>
-      </c>
-      <c r="D86" s="54"/>
+        <v>94007.791446363786</v>
+      </c>
+      <c r="D86" s="47"/>
       <c r="E86" s="9">
         <f>100-E85</f>
-        <v>16.226900729470358</v>
-      </c>
-    </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.3">
+        <v>16.52135398838827</v>
+      </c>
+    </row>
+    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B87" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="C87" s="48">
+        <v>26</v>
+      </c>
+      <c r="C87" s="41">
         <f>C84*0.03</f>
         <v>15000</v>
       </c>
-      <c r="D87" s="49"/>
+      <c r="D87" s="42"/>
       <c r="E87" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
       <c r="B88" s="27" t="s">
-        <v>28</v>
-      </c>
-      <c r="C88" s="48">
+        <v>27</v>
+      </c>
+      <c r="C88" s="41">
         <f>C84*0.02</f>
         <v>10000</v>
       </c>
-      <c r="D88" s="49"/>
+      <c r="D88" s="42"/>
       <c r="E88" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C87:D87"/>
     <mergeCell ref="C88:D88"/>
     <mergeCell ref="A7:F7"/>
@@ -3099,21 +3106,11 @@
     <mergeCell ref="C84:D84"/>
     <mergeCell ref="C85:D85"/>
     <mergeCell ref="C86:D86"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
   <headerFooter>
     <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
   </headerFooter>
-  <rowBreaks count="1" manualBreakCount="1">
-    <brk id="42" max="10" man="1"/>
-  </rowBreaks>
 </worksheet>
 </file>
</xml_diff>